<commit_message>
Major blocking bug fixes
</commit_message>
<xml_diff>
--- a/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
+++ b/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01c1829094dbd390/Desktop/Kelly_Lab/.venv/worklist_git/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/metadata_capture/excel_utils/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{E5540730-690F-444D-A5F0-1D8FDBE0762C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96077A02-DB05-4FE3-8A36-234DBAAA34D8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894E267B-80D4-554D-9651-1904BD319DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16940" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
   <si>
     <t>Number:</t>
   </si>
@@ -135,9 +135,6 @@
     <t>Experiment One</t>
   </si>
   <si>
-    <t>Either write "All" for experiment one or a number range corresponding to the Number (AD) column. For example "1-3" and "4-6".</t>
-  </si>
-  <si>
     <t>Frequency of system validation (#)</t>
   </si>
   <si>
@@ -171,12 +168,6 @@
     <t>Notebook Code:</t>
   </si>
   <si>
-    <t>A long set of instructions:</t>
-  </si>
-  <si>
-    <t>Doesn't use all wells in order to create blocks of the same size.</t>
-  </si>
-  <si>
     <t>Experiment Name:</t>
   </si>
   <si>
@@ -208,6 +199,12 @@
   </si>
   <si>
     <t>(choose)</t>
+  </si>
+  <si>
+    <t>Either write "All" for experiment one or a number range corresponding to the Number column (AD). For example, "1-5" and "6-10".</t>
+  </si>
+  <si>
+    <t>Doesn't use all wells in order to create blocks of uniform size.</t>
   </si>
 </sst>
 </file>
@@ -256,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -422,11 +419,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
@@ -487,10 +495,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -499,10 +503,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -522,6 +522,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,10 +544,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -861,7 +864,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4A45856-9C0F-D140-AD60-2AFFFFA45290}">
   <dimension ref="A1:AV63"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
@@ -884,9 +887,9 @@
     <col min="43" max="45" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2"/>
       <c r="AD1" s="5" t="s">
@@ -899,14 +902,14 @@
         <v>2</v>
       </c>
       <c r="AG1" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM1" s="34"/>
-      <c r="AO1" s="33"/>
-    </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.4">
+        <v>45</v>
+      </c>
+      <c r="AM1" s="32"/>
+      <c r="AO1" s="31"/>
+    </row>
+    <row r="2" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2"/>
       <c r="AD2" s="12">
@@ -915,19 +918,17 @@
       <c r="AE2" s="8"/>
       <c r="AF2" s="7"/>
       <c r="AG2" s="29"/>
-      <c r="AI2" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="AJ2" s="10"/>
-      <c r="AK2" s="10"/>
+      <c r="AI2" s="41"/>
+      <c r="AJ2" s="41"/>
+      <c r="AK2" s="41"/>
       <c r="AL2" s="10"/>
       <c r="AM2" s="10"/>
       <c r="AN2" s="10"/>
-      <c r="AO2" s="33"/>
-    </row>
-    <row r="3" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="AO2" s="31"/>
+    </row>
+    <row r="3" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B3" s="2"/>
       <c r="AD3" s="12">
@@ -936,19 +937,19 @@
       <c r="AE3" s="8"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="29"/>
-      <c r="AI3" s="37"/>
-      <c r="AJ3" s="10"/>
-      <c r="AK3" s="10"/>
+      <c r="AI3" s="41"/>
+      <c r="AJ3" s="41"/>
+      <c r="AK3" s="41"/>
       <c r="AL3" s="10"/>
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
-      <c r="AO3" s="33"/>
-      <c r="AU3" s="36" t="s">
+      <c r="AO3" s="31"/>
+      <c r="AU3" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="AV3" s="36"/>
-    </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AV3" s="34"/>
+    </row>
+    <row r="4" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="D4" s="3"/>
@@ -982,17 +983,17 @@
       <c r="AE4" s="8"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="29"/>
-      <c r="AI4" s="37"/>
-      <c r="AJ4" s="10"/>
-      <c r="AK4" s="10"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
       <c r="AL4" s="10"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
-      <c r="AO4" s="33"/>
-      <c r="AU4" s="36"/>
-      <c r="AV4" s="36"/>
-    </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO4" s="31"/>
+      <c r="AU4" s="34"/>
+      <c r="AV4" s="34"/>
+    </row>
+    <row r="5" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -1080,19 +1081,19 @@
       <c r="AE5" s="8"/>
       <c r="AF5" s="7"/>
       <c r="AG5" s="29"/>
-      <c r="AI5" s="37"/>
-      <c r="AJ5" s="10"/>
-      <c r="AK5" s="10"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="41"/>
       <c r="AL5" s="10"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
-      <c r="AO5" s="33"/>
-      <c r="AU5" s="36"/>
-      <c r="AV5" s="36"/>
-    </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO5" s="31"/>
+      <c r="AU5" s="34"/>
+      <c r="AV5" s="34"/>
+    </row>
+    <row r="6" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6" s="13"/>
       <c r="D6" t="s">
@@ -1128,17 +1129,17 @@
       <c r="AE6" s="8"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="29"/>
-      <c r="AI6" s="37"/>
-      <c r="AJ6" s="10"/>
-      <c r="AK6" s="10"/>
+      <c r="AI6" s="41"/>
+      <c r="AJ6" s="41"/>
+      <c r="AK6" s="41"/>
       <c r="AL6" s="10"/>
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
-      <c r="AO6" s="33"/>
-      <c r="AU6" s="36"/>
-      <c r="AV6" s="36"/>
-    </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO6" s="31"/>
+      <c r="AU6" s="34"/>
+      <c r="AV6" s="34"/>
+    </row>
+    <row r="7" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
         <v>14</v>
       </c>
@@ -1172,17 +1173,17 @@
       <c r="AE7" s="8"/>
       <c r="AF7" s="7"/>
       <c r="AG7" s="29"/>
-      <c r="AI7" s="37"/>
-      <c r="AJ7" s="10"/>
-      <c r="AK7" s="10"/>
+      <c r="AI7" s="41"/>
+      <c r="AJ7" s="41"/>
+      <c r="AK7" s="41"/>
       <c r="AL7" s="10"/>
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
-      <c r="AO7" s="33"/>
-      <c r="AU7" s="36"/>
-      <c r="AV7" s="36"/>
-    </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO7" s="31"/>
+      <c r="AU7" s="34"/>
+      <c r="AV7" s="34"/>
+    </row>
+    <row r="8" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
         <v>15</v>
       </c>
@@ -1216,17 +1217,17 @@
       <c r="AE8" s="8"/>
       <c r="AF8" s="7"/>
       <c r="AG8" s="29"/>
-      <c r="AI8" s="37"/>
-      <c r="AJ8" s="10"/>
-      <c r="AK8" s="10"/>
+      <c r="AI8" s="41"/>
+      <c r="AJ8" s="41"/>
+      <c r="AK8" s="41"/>
       <c r="AL8" s="10"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
-      <c r="AO8" s="33"/>
-      <c r="AU8" s="36"/>
-      <c r="AV8" s="36"/>
-    </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO8" s="31"/>
+      <c r="AU8" s="34"/>
+      <c r="AV8" s="34"/>
+    </row>
+    <row r="9" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D9" t="s">
         <v>16</v>
       </c>
@@ -1260,17 +1261,17 @@
       <c r="AE9" s="8"/>
       <c r="AF9" s="7"/>
       <c r="AG9" s="29"/>
-      <c r="AI9" s="37"/>
-      <c r="AJ9" s="10"/>
-      <c r="AK9" s="10"/>
+      <c r="AI9" s="41"/>
+      <c r="AJ9" s="41"/>
+      <c r="AK9" s="41"/>
       <c r="AL9" s="10"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
-      <c r="AO9" s="33"/>
-      <c r="AU9" s="36"/>
-      <c r="AV9" s="36"/>
-    </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO9" s="31"/>
+      <c r="AU9" s="34"/>
+      <c r="AV9" s="34"/>
+    </row>
+    <row r="10" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
         <v>17</v>
       </c>
@@ -1304,17 +1305,17 @@
       <c r="AE10" s="8"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="29"/>
-      <c r="AI10" s="37"/>
-      <c r="AJ10" s="10"/>
-      <c r="AK10" s="10"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="41"/>
       <c r="AL10" s="10"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
-      <c r="AO10" s="33"/>
-      <c r="AU10" s="36"/>
-      <c r="AV10" s="36"/>
-    </row>
-    <row r="11" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO10" s="31"/>
+      <c r="AU10" s="34"/>
+      <c r="AV10" s="34"/>
+    </row>
+    <row r="11" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D11" t="s">
         <v>18</v>
       </c>
@@ -1348,17 +1349,17 @@
       <c r="AE11" s="8"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="29"/>
-      <c r="AI11" s="37"/>
-      <c r="AJ11" s="10"/>
-      <c r="AK11" s="10"/>
+      <c r="AI11" s="41"/>
+      <c r="AJ11" s="41"/>
+      <c r="AK11" s="41"/>
       <c r="AL11" s="10"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
-      <c r="AO11" s="33"/>
-      <c r="AU11" s="36"/>
-      <c r="AV11" s="36"/>
-    </row>
-    <row r="12" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO11" s="31"/>
+      <c r="AU11" s="34"/>
+      <c r="AV11" s="34"/>
+    </row>
+    <row r="12" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
         <v>19</v>
       </c>
@@ -1392,17 +1393,17 @@
       <c r="AE12" s="8"/>
       <c r="AF12" s="7"/>
       <c r="AG12" s="29"/>
-      <c r="AI12" s="37"/>
-      <c r="AJ12" s="10"/>
-      <c r="AK12" s="10"/>
+      <c r="AI12" s="41"/>
+      <c r="AJ12" s="41"/>
+      <c r="AK12" s="41"/>
       <c r="AL12" s="10"/>
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
-      <c r="AO12" s="33"/>
-      <c r="AU12" s="36"/>
-      <c r="AV12" s="36"/>
-    </row>
-    <row r="13" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO12" s="31"/>
+      <c r="AU12" s="34"/>
+      <c r="AV12" s="34"/>
+    </row>
+    <row r="13" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D13" t="s">
         <v>20</v>
       </c>
@@ -1436,17 +1437,17 @@
       <c r="AE13" s="8"/>
       <c r="AF13" s="7"/>
       <c r="AG13" s="29"/>
-      <c r="AI13" s="37"/>
-      <c r="AJ13" s="10"/>
-      <c r="AK13" s="10"/>
+      <c r="AI13" s="41"/>
+      <c r="AJ13" s="41"/>
+      <c r="AK13" s="41"/>
       <c r="AL13" s="10"/>
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
-      <c r="AO13" s="33"/>
-      <c r="AU13" s="36"/>
-      <c r="AV13" s="36"/>
-    </row>
-    <row r="14" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO13" s="31"/>
+      <c r="AU13" s="34"/>
+      <c r="AV13" s="34"/>
+    </row>
+    <row r="14" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1480,17 +1481,17 @@
       <c r="AE14" s="8"/>
       <c r="AF14" s="7"/>
       <c r="AG14" s="29"/>
-      <c r="AI14" s="37"/>
-      <c r="AJ14" s="10"/>
-      <c r="AK14" s="10"/>
+      <c r="AI14" s="41"/>
+      <c r="AJ14" s="41"/>
+      <c r="AK14" s="41"/>
       <c r="AL14" s="10"/>
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
-      <c r="AO14" s="33"/>
-      <c r="AU14" s="36"/>
-      <c r="AV14" s="36"/>
-    </row>
-    <row r="15" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO14" s="31"/>
+      <c r="AU14" s="34"/>
+      <c r="AV14" s="34"/>
+    </row>
+    <row r="15" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D15" t="s">
         <v>22</v>
       </c>
@@ -1524,15 +1525,15 @@
       <c r="AE15" s="8"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="29"/>
-      <c r="AI15" s="37"/>
-      <c r="AJ15" s="10"/>
-      <c r="AK15" s="10"/>
+      <c r="AI15" s="41"/>
+      <c r="AJ15" s="41"/>
+      <c r="AK15" s="41"/>
       <c r="AL15" s="10"/>
       <c r="AM15" s="10"/>
       <c r="AN15" s="10"/>
-      <c r="AO15" s="33"/>
-    </row>
-    <row r="16" spans="1:48" x14ac:dyDescent="0.4">
+      <c r="AO15" s="31"/>
+    </row>
+    <row r="16" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
         <v>23</v>
       </c>
@@ -1566,15 +1567,15 @@
       <c r="AE16" s="8"/>
       <c r="AF16" s="7"/>
       <c r="AG16" s="29"/>
-      <c r="AI16" s="37"/>
-      <c r="AJ16" s="10"/>
-      <c r="AK16" s="10"/>
+      <c r="AI16" s="41"/>
+      <c r="AJ16" s="41"/>
+      <c r="AK16" s="41"/>
       <c r="AL16" s="10"/>
       <c r="AM16" s="10"/>
       <c r="AN16" s="10"/>
-      <c r="AO16" s="33"/>
-    </row>
-    <row r="17" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO16" s="31"/>
+    </row>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D17" t="s">
         <v>24</v>
       </c>
@@ -1608,15 +1609,15 @@
       <c r="AE17" s="8"/>
       <c r="AF17" s="7"/>
       <c r="AG17" s="29"/>
-      <c r="AI17" s="37"/>
-      <c r="AJ17" s="10"/>
-      <c r="AK17" s="10"/>
+      <c r="AI17" s="41"/>
+      <c r="AJ17" s="41"/>
+      <c r="AK17" s="41"/>
       <c r="AL17" s="10"/>
       <c r="AM17" s="10"/>
       <c r="AN17" s="10"/>
-      <c r="AO17" s="33"/>
-    </row>
-    <row r="18" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO17" s="31"/>
+    </row>
+    <row r="18" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D18" t="s">
         <v>25</v>
       </c>
@@ -1650,15 +1651,15 @@
       <c r="AE18" s="8"/>
       <c r="AF18" s="7"/>
       <c r="AG18" s="29"/>
-      <c r="AI18" s="37"/>
-      <c r="AJ18" s="10"/>
-      <c r="AK18" s="10"/>
+      <c r="AI18" s="41"/>
+      <c r="AJ18" s="41"/>
+      <c r="AK18" s="41"/>
       <c r="AL18" s="10"/>
       <c r="AM18" s="10"/>
       <c r="AN18" s="10"/>
-      <c r="AO18" s="33"/>
-    </row>
-    <row r="19" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO18" s="31"/>
+    </row>
+    <row r="19" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>26</v>
       </c>
@@ -1692,15 +1693,15 @@
       <c r="AE19" s="8"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="29"/>
-      <c r="AI19" s="37"/>
-      <c r="AJ19" s="10"/>
-      <c r="AK19" s="10"/>
+      <c r="AI19" s="41"/>
+      <c r="AJ19" s="41"/>
+      <c r="AK19" s="41"/>
       <c r="AL19" s="10"/>
       <c r="AM19" s="10"/>
       <c r="AN19" s="10"/>
-      <c r="AO19" s="33"/>
-    </row>
-    <row r="20" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO19" s="31"/>
+    </row>
+    <row r="20" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
         <v>27</v>
       </c>
@@ -1734,15 +1735,15 @@
       <c r="AE20" s="8"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="29"/>
-      <c r="AI20" s="37"/>
-      <c r="AJ20" s="10"/>
-      <c r="AK20" s="10"/>
+      <c r="AI20" s="41"/>
+      <c r="AJ20" s="41"/>
+      <c r="AK20" s="41"/>
       <c r="AL20" s="10"/>
       <c r="AM20" s="10"/>
       <c r="AN20" s="10"/>
-      <c r="AO20" s="33"/>
-    </row>
-    <row r="21" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO20" s="31"/>
+    </row>
+    <row r="21" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D21" t="s">
         <v>28</v>
       </c>
@@ -1776,15 +1777,15 @@
       <c r="AE21" s="8"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="29"/>
-      <c r="AI21" s="37"/>
-      <c r="AJ21" s="10"/>
-      <c r="AK21" s="10"/>
+      <c r="AI21" s="41"/>
+      <c r="AJ21" s="41"/>
+      <c r="AK21" s="41"/>
       <c r="AL21" s="10"/>
       <c r="AM21" s="10"/>
       <c r="AN21" s="10"/>
-      <c r="AO21" s="33"/>
-    </row>
-    <row r="22" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO21" s="31"/>
+    </row>
+    <row r="22" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="D22" s="3"/>
@@ -1818,15 +1819,15 @@
       <c r="AE22" s="8"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="29"/>
-      <c r="AI22" s="37"/>
-      <c r="AJ22" s="10"/>
-      <c r="AK22" s="10"/>
+      <c r="AI22" s="41"/>
+      <c r="AJ22" s="41"/>
+      <c r="AK22" s="41"/>
       <c r="AL22" s="10"/>
       <c r="AM22" s="10"/>
       <c r="AN22" s="10"/>
-      <c r="AO22" s="33"/>
-    </row>
-    <row r="23" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO22" s="31"/>
+    </row>
+    <row r="23" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>10</v>
       </c>
@@ -1914,15 +1915,15 @@
       <c r="AE23" s="8"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="29"/>
-      <c r="AI23" s="37"/>
-      <c r="AJ23" s="10"/>
-      <c r="AK23" s="10"/>
+      <c r="AI23" s="41"/>
+      <c r="AJ23" s="41"/>
+      <c r="AK23" s="41"/>
       <c r="AL23" s="10"/>
       <c r="AM23" s="10"/>
       <c r="AN23" s="10"/>
-      <c r="AO23" s="33"/>
-    </row>
-    <row r="24" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO23" s="31"/>
+    </row>
+    <row r="24" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>19</v>
       </c>
@@ -1960,15 +1961,15 @@
       <c r="AE24" s="8"/>
       <c r="AF24" s="7"/>
       <c r="AG24" s="29"/>
-      <c r="AI24" s="37"/>
-      <c r="AJ24" s="10"/>
-      <c r="AK24" s="10"/>
+      <c r="AI24" s="41"/>
+      <c r="AJ24" s="41"/>
+      <c r="AK24" s="41"/>
       <c r="AL24" s="10"/>
       <c r="AM24" s="10"/>
       <c r="AN24" s="10"/>
-      <c r="AO24" s="33"/>
-    </row>
-    <row r="25" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO24" s="31"/>
+    </row>
+    <row r="25" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D25" t="s">
         <v>14</v>
       </c>
@@ -2002,15 +2003,15 @@
       <c r="AE25" s="8"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="29"/>
-      <c r="AI25" s="37"/>
-      <c r="AJ25" s="10"/>
-      <c r="AK25" s="10"/>
+      <c r="AI25" s="41"/>
+      <c r="AJ25" s="41"/>
+      <c r="AK25" s="41"/>
       <c r="AL25" s="10"/>
       <c r="AM25" s="10"/>
       <c r="AN25" s="10"/>
-      <c r="AO25" s="33"/>
-    </row>
-    <row r="26" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO25" s="31"/>
+    </row>
+    <row r="26" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D26" t="s">
         <v>15</v>
       </c>
@@ -2044,15 +2045,15 @@
       <c r="AE26" s="8"/>
       <c r="AF26" s="7"/>
       <c r="AG26" s="29"/>
-      <c r="AI26" s="37"/>
-      <c r="AJ26" s="10"/>
-      <c r="AK26" s="10"/>
+      <c r="AI26" s="41"/>
+      <c r="AJ26" s="41"/>
+      <c r="AK26" s="41"/>
       <c r="AL26" s="10"/>
       <c r="AM26" s="10"/>
       <c r="AN26" s="10"/>
-      <c r="AO26" s="33"/>
-    </row>
-    <row r="27" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO26" s="31"/>
+    </row>
+    <row r="27" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D27" t="s">
         <v>16</v>
       </c>
@@ -2086,15 +2087,15 @@
       <c r="AE27" s="8"/>
       <c r="AF27" s="7"/>
       <c r="AG27" s="29"/>
-      <c r="AI27" s="37"/>
-      <c r="AJ27" s="10"/>
-      <c r="AK27" s="10"/>
+      <c r="AI27" s="41"/>
+      <c r="AJ27" s="41"/>
+      <c r="AK27" s="41"/>
       <c r="AL27" s="10"/>
       <c r="AM27" s="10"/>
       <c r="AN27" s="10"/>
-      <c r="AO27" s="33"/>
-    </row>
-    <row r="28" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO27" s="31"/>
+    </row>
+    <row r="28" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D28" t="s">
         <v>17</v>
       </c>
@@ -2128,15 +2129,15 @@
       <c r="AE28" s="8"/>
       <c r="AF28" s="7"/>
       <c r="AG28" s="29"/>
-      <c r="AI28" s="37"/>
-      <c r="AJ28" s="10"/>
-      <c r="AK28" s="10"/>
+      <c r="AI28" s="41"/>
+      <c r="AJ28" s="41"/>
+      <c r="AK28" s="41"/>
       <c r="AL28" s="10"/>
       <c r="AM28" s="10"/>
       <c r="AN28" s="10"/>
-      <c r="AO28" s="33"/>
-    </row>
-    <row r="29" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO28" s="31"/>
+    </row>
+    <row r="29" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D29" t="s">
         <v>18</v>
       </c>
@@ -2170,15 +2171,15 @@
       <c r="AE29" s="8"/>
       <c r="AF29" s="7"/>
       <c r="AG29" s="29"/>
-      <c r="AI29" s="37"/>
-      <c r="AJ29" s="10"/>
-      <c r="AK29" s="10"/>
+      <c r="AI29" s="41"/>
+      <c r="AJ29" s="41"/>
+      <c r="AK29" s="41"/>
       <c r="AL29" s="10"/>
       <c r="AM29" s="10"/>
       <c r="AN29" s="10"/>
-      <c r="AO29" s="33"/>
-    </row>
-    <row r="30" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO29" s="31"/>
+    </row>
+    <row r="30" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D30" t="s">
         <v>19</v>
       </c>
@@ -2212,15 +2213,15 @@
       <c r="AE30" s="8"/>
       <c r="AF30" s="7"/>
       <c r="AG30" s="29"/>
-      <c r="AI30" s="37"/>
-      <c r="AJ30" s="10"/>
-      <c r="AK30" s="10"/>
+      <c r="AI30" s="41"/>
+      <c r="AJ30" s="41"/>
+      <c r="AK30" s="41"/>
       <c r="AL30" s="10"/>
       <c r="AM30" s="10"/>
       <c r="AN30" s="10"/>
-      <c r="AO30" s="33"/>
-    </row>
-    <row r="31" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO30" s="31"/>
+    </row>
+    <row r="31" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D31" t="s">
         <v>20</v>
       </c>
@@ -2254,15 +2255,15 @@
       <c r="AE31" s="8"/>
       <c r="AF31" s="7"/>
       <c r="AG31" s="29"/>
-      <c r="AI31" s="37"/>
-      <c r="AJ31" s="10"/>
-      <c r="AK31" s="10"/>
+      <c r="AI31" s="41"/>
+      <c r="AJ31" s="41"/>
+      <c r="AK31" s="41"/>
       <c r="AL31" s="10"/>
       <c r="AM31" s="10"/>
       <c r="AN31" s="10"/>
-      <c r="AO31" s="33"/>
-    </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO31" s="31"/>
+    </row>
+    <row r="32" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D32" t="s">
         <v>21</v>
       </c>
@@ -2302,9 +2303,9 @@
       <c r="AL32" s="10"/>
       <c r="AM32" s="10"/>
       <c r="AN32" s="10"/>
-      <c r="AO32" s="33"/>
-    </row>
-    <row r="33" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="AO32" s="31"/>
+    </row>
+    <row r="33" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D33" t="s">
         <v>22</v>
       </c>
@@ -2339,20 +2340,20 @@
       <c r="AF33" s="7"/>
       <c r="AG33" s="29"/>
       <c r="AI33" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AJ33" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="AK33" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="AL33" s="43"/>
+        <v>35</v>
+      </c>
+      <c r="AK33" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL33" s="40"/>
       <c r="AM33" s="10"/>
       <c r="AN33" s="10"/>
-      <c r="AO33" s="33"/>
-    </row>
-    <row r="34" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AO33" s="31"/>
+    </row>
+    <row r="34" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D34" t="s">
         <v>23</v>
       </c>
@@ -2386,13 +2387,14 @@
       <c r="AE34" s="12"/>
       <c r="AF34" s="11"/>
       <c r="AG34" s="11"/>
-      <c r="AI34" t="s">
-        <v>55</v>
-      </c>
-      <c r="AK34" s="43"/>
-      <c r="AL34" s="43"/>
-    </row>
-    <row r="35" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="AI34" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ34" s="6"/>
+      <c r="AK34" s="23"/>
+      <c r="AL34" s="23"/>
+    </row>
+    <row r="35" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
         <v>24</v>
       </c>
@@ -2428,7 +2430,7 @@
       <c r="AG35" s="11"/>
       <c r="AK35" s="23"/>
     </row>
-    <row r="36" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
         <v>25</v>
       </c>
@@ -2466,14 +2468,14 @@
         <v>31</v>
       </c>
       <c r="AJ36" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK36" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="AL36" s="43"/>
-    </row>
-    <row r="37" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+      <c r="AK36" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL36" s="40"/>
+    </row>
+    <row r="37" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D37" t="s">
         <v>26</v>
       </c>
@@ -2508,13 +2510,13 @@
       <c r="AF37" s="11"/>
       <c r="AG37" s="11"/>
       <c r="AI37" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AJ37" s="6"/>
-      <c r="AK37" s="42"/>
-      <c r="AL37" s="43"/>
-    </row>
-    <row r="38" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="AK37" s="39"/>
+      <c r="AL37" s="40"/>
+    </row>
+    <row r="38" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D38" t="s">
         <v>27</v>
       </c>
@@ -2548,16 +2550,16 @@
       <c r="AE38" s="12"/>
       <c r="AF38" s="11"/>
       <c r="AG38" s="11"/>
-      <c r="AI38" s="38" t="s">
+      <c r="AI38" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ38" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="AJ38" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="AK38" s="42"/>
-      <c r="AL38" s="43"/>
-    </row>
-    <row r="39" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AK38" s="39"/>
+      <c r="AL38" s="40"/>
+    </row>
+    <row r="39" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D39" t="s">
         <v>28</v>
       </c>
@@ -2591,12 +2593,12 @@
       <c r="AE39" s="12"/>
       <c r="AF39" s="11"/>
       <c r="AG39" s="11"/>
-      <c r="AI39" s="39"/>
-      <c r="AJ39" s="41"/>
-      <c r="AK39" s="35"/>
-      <c r="AL39" s="35"/>
-    </row>
-    <row r="40" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AI39" s="36"/>
+      <c r="AJ39" s="38"/>
+      <c r="AK39" s="33"/>
+      <c r="AL39" s="33"/>
+    </row>
+    <row r="40" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="D40" s="3"/>
@@ -2630,10 +2632,10 @@
       <c r="AE40" s="12"/>
       <c r="AF40" s="11"/>
       <c r="AG40" s="11"/>
-      <c r="AJ40" s="35"/>
-      <c r="AK40" s="35"/>
-    </row>
-    <row r="41" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AJ40" s="33"/>
+      <c r="AK40" s="33"/>
+    </row>
+    <row r="41" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>10</v>
       </c>
@@ -2641,7 +2643,7 @@
         <v>11</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2721,10 +2723,10 @@
       <c r="AE41" s="12"/>
       <c r="AF41" s="11"/>
       <c r="AG41" s="11"/>
-      <c r="AJ41" s="35"/>
-      <c r="AK41" s="35"/>
-    </row>
-    <row r="42" spans="1:41" x14ac:dyDescent="0.4">
+      <c r="AJ41" s="33"/>
+      <c r="AK41" s="33"/>
+    </row>
+    <row r="42" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A42" s="13" t="s">
         <v>14</v>
       </c>
@@ -2763,7 +2765,7 @@
       <c r="AF42" s="11"/>
       <c r="AG42" s="11"/>
     </row>
-    <row r="43" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D43" t="s">
         <v>14</v>
       </c>
@@ -2798,7 +2800,7 @@
       <c r="AF43" s="11"/>
       <c r="AG43" s="11"/>
     </row>
-    <row r="44" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D44" t="s">
         <v>15</v>
       </c>
@@ -2833,7 +2835,7 @@
       <c r="AF44" s="11"/>
       <c r="AG44" s="11"/>
     </row>
-    <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D45" t="s">
         <v>16</v>
       </c>
@@ -2868,7 +2870,7 @@
       <c r="AF45" s="11"/>
       <c r="AG45" s="11"/>
     </row>
-    <row r="46" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D46" t="s">
         <v>17</v>
       </c>
@@ -2903,7 +2905,7 @@
       <c r="AF46" s="11"/>
       <c r="AG46" s="11"/>
     </row>
-    <row r="47" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D47" t="s">
         <v>18</v>
       </c>
@@ -2938,7 +2940,7 @@
       <c r="AF47" s="11"/>
       <c r="AG47" s="11"/>
     </row>
-    <row r="48" spans="1:41" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:41" x14ac:dyDescent="0.2">
       <c r="D48" t="s">
         <v>19</v>
       </c>
@@ -2973,7 +2975,7 @@
       <c r="AF48" s="27"/>
       <c r="AG48" s="11"/>
     </row>
-    <row r="49" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D49" t="s">
         <v>20</v>
       </c>
@@ -3008,7 +3010,7 @@
       <c r="AF49" s="27"/>
       <c r="AG49" s="11"/>
     </row>
-    <row r="50" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D50" t="s">
         <v>21</v>
       </c>
@@ -3043,7 +3045,7 @@
       <c r="AF50" s="27"/>
       <c r="AG50" s="11"/>
     </row>
-    <row r="51" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D51" t="s">
         <v>22</v>
       </c>
@@ -3078,7 +3080,7 @@
       <c r="AF51" s="21"/>
       <c r="AG51" s="21"/>
     </row>
-    <row r="52" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
         <v>23</v>
       </c>
@@ -3107,7 +3109,7 @@
       <c r="AA52" s="10"/>
       <c r="AB52" s="9"/>
     </row>
-    <row r="53" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D53" t="s">
         <v>24</v>
       </c>
@@ -3140,7 +3142,7 @@
       <c r="AM53" s="23"/>
       <c r="AN53" s="23"/>
     </row>
-    <row r="54" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D54" t="s">
         <v>25</v>
       </c>
@@ -3173,7 +3175,7 @@
       <c r="AM54" s="23"/>
       <c r="AN54" s="23"/>
     </row>
-    <row r="55" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D55" t="s">
         <v>26</v>
       </c>
@@ -3206,7 +3208,7 @@
       <c r="AM55" s="23"/>
       <c r="AN55" s="23"/>
     </row>
-    <row r="56" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:40" x14ac:dyDescent="0.2">
       <c r="D56" t="s">
         <v>27</v>
       </c>
@@ -3236,7 +3238,7 @@
       <c r="AB56" s="9"/>
       <c r="AE56" s="10"/>
     </row>
-    <row r="57" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D57" t="s">
         <v>28</v>
       </c>
@@ -3270,7 +3272,7 @@
       <c r="AM57" s="23"/>
       <c r="AN57" s="23"/>
     </row>
-    <row r="58" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="D58" s="3"/>
@@ -3304,34 +3306,33 @@
       <c r="AM58" s="23"/>
       <c r="AN58" s="23"/>
     </row>
-    <row r="59" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:40" x14ac:dyDescent="0.2">
       <c r="AE59" s="10"/>
       <c r="AK59" s="23"/>
       <c r="AL59" s="24"/>
       <c r="AM59" s="23"/>
       <c r="AN59" s="23"/>
     </row>
-    <row r="60" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:40" x14ac:dyDescent="0.2">
       <c r="AE60" s="10"/>
     </row>
-    <row r="61" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:40" x14ac:dyDescent="0.2">
       <c r="AE61" s="10"/>
     </row>
-    <row r="62" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:40" x14ac:dyDescent="0.2">
       <c r="AE62" s="10"/>
     </row>
-    <row r="63" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:40" x14ac:dyDescent="0.2">
       <c r="AE63" s="10"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="AU3:AV14"/>
-    <mergeCell ref="AI2:AI31"/>
     <mergeCell ref="AI38:AI39"/>
     <mergeCell ref="AJ38:AJ39"/>
     <mergeCell ref="AK36:AL38"/>
-    <mergeCell ref="AK33:AL34"/>
+    <mergeCell ref="AK33:AL33"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="3">
@@ -3353,14 +3354,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA40715-6F6B-5649-8058-60881427272C}">
   <dimension ref="A1:R51"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="17" max="17" width="29.33203125" customWidth="1"/>
     <col min="18" max="18" width="24.6640625" customWidth="1"/>
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3370,7 +3371,7 @@
       <c r="C1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
@@ -3380,7 +3381,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>6</v>
@@ -3392,25 +3393,25 @@
         <v>8</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L1" s="28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -3422,7 +3423,7 @@
         <f>IF(LEN(User!AF2)=0,"",User!AF2)</f>
         <v/>
       </c>
-      <c r="D2" s="9"/>
+      <c r="D2" s="7"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="7"/>
@@ -3437,14 +3438,15 @@
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
       <c r="O2" s="11"/>
-      <c r="Q2" s="1" t="s">
-        <v>47</v>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="42" t="s">
+        <v>44</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.4">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -3456,7 +3458,7 @@
         <f>IF(LEN(User!AF3)=0,"",User!AF3)</f>
         <v/>
       </c>
-      <c r="D3" s="9"/>
+      <c r="D3" s="7"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="7"/>
@@ -3471,8 +3473,9 @@
       <c r="M3" s="12"/>
       <c r="N3" s="12"/>
       <c r="O3" s="11"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P3" s="11"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -3484,7 +3487,7 @@
         <f>IF(LEN(User!AF4)=0,"",User!AF4)</f>
         <v/>
       </c>
-      <c r="D4" s="9"/>
+      <c r="D4" s="7"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
       <c r="G4" s="7"/>
@@ -3499,10 +3502,11 @@
       <c r="M4" s="12"/>
       <c r="N4" s="12"/>
       <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
       <c r="Q4" s="23"/>
       <c r="R4" s="24"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -3514,7 +3518,7 @@
         <f>IF(LEN(User!AF5)=0,"",User!AF5)</f>
         <v/>
       </c>
-      <c r="D5" s="9"/>
+      <c r="D5" s="7"/>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="7"/>
@@ -3529,14 +3533,15 @@
       <c r="M5" s="12"/>
       <c r="N5" s="12"/>
       <c r="O5" s="11"/>
-      <c r="Q5" s="1" t="s">
-        <v>49</v>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="42" t="s">
+        <v>46</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.4">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -3548,7 +3553,7 @@
         <f>IF(LEN(User!AF6)=0,"",User!AF6)</f>
         <v/>
       </c>
-      <c r="D6" s="9"/>
+      <c r="D6" s="7"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="7"/>
@@ -3563,12 +3568,13 @@
       <c r="M6" s="12"/>
       <c r="N6" s="12"/>
       <c r="O6" s="11"/>
-      <c r="Q6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="R6" s="32"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P6" s="11"/>
+      <c r="Q6" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="R6" s="30"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -3580,7 +3586,7 @@
         <f>IF(LEN(User!AF7)=0,"",User!AF7)</f>
         <v/>
       </c>
-      <c r="D7" s="9"/>
+      <c r="D7" s="7"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="7"/>
@@ -3595,14 +3601,15 @@
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
       <c r="O7" s="11"/>
-      <c r="Q7" s="1" t="s">
-        <v>52</v>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="42" t="s">
+        <v>49</v>
       </c>
       <c r="R7" s="6">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -3614,7 +3621,7 @@
         <f>IF(LEN(User!AF8)=0,"",User!AF8)</f>
         <v/>
       </c>
-      <c r="D8" s="9"/>
+      <c r="D8" s="7"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="7"/>
@@ -3629,8 +3636,9 @@
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
       <c r="O8" s="11"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P8" s="11"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -3642,7 +3650,7 @@
         <f>IF(LEN(User!AF9)=0,"",User!AF9)</f>
         <v/>
       </c>
-      <c r="D9" s="9"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="7"/>
@@ -3657,8 +3665,9 @@
       <c r="M9" s="12"/>
       <c r="N9" s="12"/>
       <c r="O9" s="11"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P9" s="11"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -3670,7 +3679,7 @@
         <f>IF(LEN(User!AF10)=0,"",User!AF10)</f>
         <v/>
       </c>
-      <c r="D10" s="9"/>
+      <c r="D10" s="7"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="7"/>
@@ -3685,8 +3694,9 @@
       <c r="M10" s="12"/>
       <c r="N10" s="12"/>
       <c r="O10" s="11"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P10" s="11"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="12">
         <v>10</v>
       </c>
@@ -3698,7 +3708,7 @@
         <f>IF(LEN(User!AF11)=0,"",User!AF11)</f>
         <v/>
       </c>
-      <c r="D11" s="9"/>
+      <c r="D11" s="7"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11" s="7"/>
@@ -3713,8 +3723,9 @@
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
       <c r="O11" s="11"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P11" s="11"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -3726,7 +3737,7 @@
         <f>IF(LEN(User!AF12)=0,"",User!AF12)</f>
         <v/>
       </c>
-      <c r="D12" s="9"/>
+      <c r="D12" s="7"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
       <c r="G12" s="7"/>
@@ -3741,8 +3752,9 @@
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
       <c r="O12" s="11"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P12" s="11"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -3754,7 +3766,7 @@
         <f>IF(LEN(User!AF13)=0,"",User!AF13)</f>
         <v/>
       </c>
-      <c r="D13" s="9"/>
+      <c r="D13" s="7"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
       <c r="G13" s="7"/>
@@ -3769,8 +3781,9 @@
       <c r="M13" s="12"/>
       <c r="N13" s="12"/>
       <c r="O13" s="11"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P13" s="11"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -3782,7 +3795,7 @@
         <f>IF(LEN(User!AF14)=0,"",User!AF14)</f>
         <v/>
       </c>
-      <c r="D14" s="9"/>
+      <c r="D14" s="7"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
       <c r="G14" s="7"/>
@@ -3797,8 +3810,9 @@
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
       <c r="O14" s="11"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="P14" s="11"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -3810,7 +3824,7 @@
         <f>IF(LEN(User!AF15)=0,"",User!AF15)</f>
         <v/>
       </c>
-      <c r="D15" s="9"/>
+      <c r="D15" s="7"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
       <c r="G15" s="7"/>
@@ -3825,8 +3839,9 @@
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
       <c r="O15" s="11"/>
-    </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -3838,7 +3853,7 @@
         <f>IF(LEN(User!AF16)=0,"",User!AF16)</f>
         <v/>
       </c>
-      <c r="D16" s="9"/>
+      <c r="D16" s="7"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="7"/>
@@ -3853,8 +3868,9 @@
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
       <c r="O16" s="11"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P16" s="11"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -3866,7 +3882,7 @@
         <f>IF(LEN(User!AF17)=0,"",User!AF17)</f>
         <v/>
       </c>
-      <c r="D17" s="9"/>
+      <c r="D17" s="7"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
       <c r="G17" s="7"/>
@@ -3881,8 +3897,9 @@
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
       <c r="O17" s="11"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P17" s="11"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="12">
         <v>17</v>
       </c>
@@ -3894,7 +3911,7 @@
         <f>IF(LEN(User!AF18)=0,"",User!AF18)</f>
         <v/>
       </c>
-      <c r="D18" s="9"/>
+      <c r="D18" s="7"/>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
       <c r="G18" s="7"/>
@@ -3909,8 +3926,9 @@
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
       <c r="O18" s="11"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="12">
         <v>18</v>
       </c>
@@ -3922,7 +3940,7 @@
         <f>IF(LEN(User!AF19)=0,"",User!AF19)</f>
         <v/>
       </c>
-      <c r="D19" s="9"/>
+      <c r="D19" s="7"/>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
       <c r="G19" s="7"/>
@@ -3937,8 +3955,9 @@
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
       <c r="O19" s="11"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P19" s="11"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="12">
         <v>19</v>
       </c>
@@ -3950,7 +3969,7 @@
         <f>IF(LEN(User!AF20)=0,"",User!AF20)</f>
         <v/>
       </c>
-      <c r="D20" s="9"/>
+      <c r="D20" s="7"/>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
       <c r="G20" s="7"/>
@@ -3965,8 +3984,9 @@
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
       <c r="O20" s="11"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P20" s="11"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" s="12">
         <v>20</v>
       </c>
@@ -3978,7 +3998,7 @@
         <f>IF(LEN(User!AF21)=0,"",User!AF21)</f>
         <v/>
       </c>
-      <c r="D21" s="9"/>
+      <c r="D21" s="7"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="7"/>
@@ -3993,8 +4013,9 @@
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
       <c r="O21" s="11"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P21" s="11"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="12">
         <v>21</v>
       </c>
@@ -4006,7 +4027,7 @@
         <f>IF(LEN(User!AF22)=0,"",User!AF22)</f>
         <v/>
       </c>
-      <c r="D22" s="9"/>
+      <c r="D22" s="7"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="7"/>
@@ -4021,8 +4042,9 @@
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="11"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P22" s="11"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="12">
         <v>22</v>
       </c>
@@ -4034,7 +4056,7 @@
         <f>IF(LEN(User!AF23)=0,"",User!AF23)</f>
         <v/>
       </c>
-      <c r="D23" s="9"/>
+      <c r="D23" s="7"/>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
       <c r="G23" s="7"/>
@@ -4049,8 +4071,9 @@
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
       <c r="O23" s="11"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P23" s="11"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -4062,7 +4085,7 @@
         <f>IF(LEN(User!AF24)=0,"",User!AF24)</f>
         <v/>
       </c>
-      <c r="D24" s="9"/>
+      <c r="D24" s="7"/>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
       <c r="G24" s="7"/>
@@ -4077,8 +4100,9 @@
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
       <c r="O24" s="11"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P24" s="11"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -4090,7 +4114,7 @@
         <f>IF(LEN(User!AF25)=0,"",User!AF25)</f>
         <v/>
       </c>
-      <c r="D25" s="9"/>
+      <c r="D25" s="7"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
       <c r="G25" s="7"/>
@@ -4105,8 +4129,9 @@
       <c r="M25" s="12"/>
       <c r="N25" s="12"/>
       <c r="O25" s="11"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P25" s="11"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="12">
         <v>25</v>
       </c>
@@ -4118,7 +4143,7 @@
         <f>IF(LEN(User!AF26)=0,"",User!AF26)</f>
         <v/>
       </c>
-      <c r="D26" s="9"/>
+      <c r="D26" s="7"/>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
       <c r="G26" s="7"/>
@@ -4133,8 +4158,9 @@
       <c r="M26" s="12"/>
       <c r="N26" s="12"/>
       <c r="O26" s="11"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P26" s="11"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="12">
         <v>26</v>
       </c>
@@ -4146,7 +4172,7 @@
         <f>IF(LEN(User!AF27)=0,"",User!AF27)</f>
         <v/>
       </c>
-      <c r="D27" s="9"/>
+      <c r="D27" s="7"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
       <c r="G27" s="7"/>
@@ -4161,8 +4187,9 @@
       <c r="M27" s="12"/>
       <c r="N27" s="12"/>
       <c r="O27" s="11"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P27" s="11"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="12">
         <v>27</v>
       </c>
@@ -4174,7 +4201,7 @@
         <f>IF(LEN(User!AF28)=0,"",User!AF28)</f>
         <v/>
       </c>
-      <c r="D28" s="9"/>
+      <c r="D28" s="7"/>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
       <c r="G28" s="7"/>
@@ -4189,8 +4216,9 @@
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
       <c r="O28" s="11"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P28" s="11"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -4202,7 +4230,7 @@
         <f>IF(LEN(User!AF29)=0,"",User!AF29)</f>
         <v/>
       </c>
-      <c r="D29" s="9"/>
+      <c r="D29" s="7"/>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
       <c r="G29" s="7"/>
@@ -4217,8 +4245,9 @@
       <c r="M29" s="12"/>
       <c r="N29" s="12"/>
       <c r="O29" s="11"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P29" s="11"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="12">
         <v>29</v>
       </c>
@@ -4230,7 +4259,7 @@
         <f>IF(LEN(User!AF30)=0,"",User!AF30)</f>
         <v/>
       </c>
-      <c r="D30" s="9"/>
+      <c r="D30" s="7"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
       <c r="G30" s="7"/>
@@ -4245,8 +4274,9 @@
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
       <c r="O30" s="11"/>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P30" s="11"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="12">
         <v>30</v>
       </c>
@@ -4258,7 +4288,7 @@
         <f>IF(LEN(User!AF31)=0,"",User!AF31)</f>
         <v/>
       </c>
-      <c r="D31" s="9"/>
+      <c r="D31" s="7"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
       <c r="G31" s="7"/>
@@ -4273,8 +4303,9 @@
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
       <c r="O31" s="11"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P31" s="11"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" s="12">
         <v>31</v>
       </c>
@@ -4286,7 +4317,7 @@
         <f>IF(LEN(User!AF32)=0,"",User!AF32)</f>
         <v/>
       </c>
-      <c r="D32" s="9"/>
+      <c r="D32" s="7"/>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
       <c r="G32" s="7"/>
@@ -4301,8 +4332,9 @@
       <c r="M32" s="12"/>
       <c r="N32" s="12"/>
       <c r="O32" s="11"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P32" s="11"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" s="12">
         <v>32</v>
       </c>
@@ -4314,7 +4346,7 @@
         <f>IF(LEN(User!AF33)=0,"",User!AF33)</f>
         <v/>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="7"/>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
       <c r="G33" s="7"/>
@@ -4329,8 +4361,9 @@
       <c r="M33" s="12"/>
       <c r="N33" s="12"/>
       <c r="O33" s="11"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P33" s="11"/>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" s="12">
         <v>33</v>
       </c>
@@ -4342,7 +4375,7 @@
         <f>IF(LEN(User!AF34)=0,"",User!AF34)</f>
         <v/>
       </c>
-      <c r="D34" s="30"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="12"/>
       <c r="F34" s="12"/>
       <c r="G34" s="11"/>
@@ -4357,8 +4390,9 @@
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
       <c r="O34" s="11"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P34" s="11"/>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" s="12">
         <v>34</v>
       </c>
@@ -4370,7 +4404,7 @@
         <f>IF(LEN(User!AF35)=0,"",User!AF35)</f>
         <v/>
       </c>
-      <c r="D35" s="30"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
       <c r="G35" s="11"/>
@@ -4385,8 +4419,9 @@
       <c r="M35" s="12"/>
       <c r="N35" s="12"/>
       <c r="O35" s="11"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P35" s="11"/>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" s="12">
         <v>35</v>
       </c>
@@ -4398,7 +4433,7 @@
         <f>IF(LEN(User!AF36)=0,"",User!AF36)</f>
         <v/>
       </c>
-      <c r="D36" s="30"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
       <c r="G36" s="11"/>
@@ -4412,8 +4447,9 @@
       </c>
       <c r="N36" s="12"/>
       <c r="O36" s="11"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P36" s="11"/>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" s="12">
         <v>36</v>
       </c>
@@ -4425,7 +4461,7 @@
         <f>IF(LEN(User!AF37)=0,"",User!AF37)</f>
         <v/>
       </c>
-      <c r="D37" s="30"/>
+      <c r="D37" s="11"/>
       <c r="E37" s="12"/>
       <c r="F37" s="12"/>
       <c r="G37" s="11"/>
@@ -4440,8 +4476,9 @@
       <c r="M37" s="12"/>
       <c r="N37" s="12"/>
       <c r="O37" s="11"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P37" s="11"/>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" s="12">
         <v>37</v>
       </c>
@@ -4453,7 +4490,7 @@
         <f>IF(LEN(User!AF38)=0,"",User!AF38)</f>
         <v/>
       </c>
-      <c r="D38" s="30"/>
+      <c r="D38" s="11"/>
       <c r="E38" s="12"/>
       <c r="F38" s="12"/>
       <c r="G38" s="11"/>
@@ -4468,8 +4505,9 @@
       <c r="M38" s="12"/>
       <c r="N38" s="12"/>
       <c r="O38" s="11"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P38" s="11"/>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" s="12">
         <v>38</v>
       </c>
@@ -4481,7 +4519,7 @@
         <f>IF(LEN(User!AF39)=0,"",User!AF39)</f>
         <v/>
       </c>
-      <c r="D39" s="30"/>
+      <c r="D39" s="11"/>
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
       <c r="G39" s="11"/>
@@ -4496,8 +4534,9 @@
       <c r="M39" s="12"/>
       <c r="N39" s="12"/>
       <c r="O39" s="11"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P39" s="11"/>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" s="12">
         <v>39</v>
       </c>
@@ -4509,7 +4548,7 @@
         <f>IF(LEN(User!AF40)=0,"",User!AF40)</f>
         <v/>
       </c>
-      <c r="D40" s="30"/>
+      <c r="D40" s="11"/>
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
       <c r="G40" s="11"/>
@@ -4524,8 +4563,9 @@
       <c r="M40" s="12"/>
       <c r="N40" s="12"/>
       <c r="O40" s="11"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P40" s="11"/>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" s="12">
         <v>40</v>
       </c>
@@ -4537,7 +4577,7 @@
         <f>IF(LEN(User!AF41)=0,"",User!AF41)</f>
         <v/>
       </c>
-      <c r="D41" s="30"/>
+      <c r="D41" s="11"/>
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
       <c r="G41" s="11"/>
@@ -4552,8 +4592,9 @@
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
       <c r="O41" s="11"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P41" s="11"/>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="12">
         <v>41</v>
       </c>
@@ -4565,7 +4606,7 @@
         <f>IF(LEN(User!AF42)=0,"",User!AF42)</f>
         <v/>
       </c>
-      <c r="D42" s="30"/>
+      <c r="D42" s="11"/>
       <c r="E42" s="12"/>
       <c r="F42" s="12"/>
       <c r="G42" s="11"/>
@@ -4580,8 +4621,9 @@
       <c r="M42" s="12"/>
       <c r="N42" s="12"/>
       <c r="O42" s="11"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P42" s="11"/>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" s="12">
         <v>42</v>
       </c>
@@ -4593,7 +4635,7 @@
         <f>IF(LEN(User!AF43)=0,"",User!AF43)</f>
         <v/>
       </c>
-      <c r="D43" s="30"/>
+      <c r="D43" s="11"/>
       <c r="E43" s="12"/>
       <c r="F43" s="12"/>
       <c r="G43" s="11"/>
@@ -4608,8 +4650,9 @@
       <c r="M43" s="12"/>
       <c r="N43" s="12"/>
       <c r="O43" s="11"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P43" s="11"/>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="12">
         <v>43</v>
       </c>
@@ -4621,7 +4664,7 @@
         <f>IF(LEN(User!AF44)=0,"",User!AF44)</f>
         <v/>
       </c>
-      <c r="D44" s="30"/>
+      <c r="D44" s="11"/>
       <c r="E44" s="12"/>
       <c r="F44" s="12"/>
       <c r="G44" s="11"/>
@@ -4636,8 +4679,9 @@
       <c r="M44" s="12"/>
       <c r="N44" s="12"/>
       <c r="O44" s="11"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P44" s="11"/>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" s="12">
         <v>44</v>
       </c>
@@ -4649,7 +4693,7 @@
         <f>IF(LEN(User!AF45)=0,"",User!AF45)</f>
         <v/>
       </c>
-      <c r="D45" s="30"/>
+      <c r="D45" s="11"/>
       <c r="E45" s="12"/>
       <c r="F45" s="12"/>
       <c r="G45" s="11"/>
@@ -4664,8 +4708,9 @@
       <c r="M45" s="12"/>
       <c r="N45" s="12"/>
       <c r="O45" s="11"/>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P45" s="11"/>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="12">
         <v>45</v>
       </c>
@@ -4677,7 +4722,7 @@
         <f>IF(LEN(User!AF46)=0,"",User!AF46)</f>
         <v/>
       </c>
-      <c r="D46" s="30"/>
+      <c r="D46" s="11"/>
       <c r="E46" s="12"/>
       <c r="F46" s="12"/>
       <c r="G46" s="11"/>
@@ -4692,8 +4737,9 @@
       <c r="M46" s="12"/>
       <c r="N46" s="12"/>
       <c r="O46" s="11"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P46" s="11"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" s="12">
         <v>46</v>
       </c>
@@ -4705,7 +4751,7 @@
         <f>IF(LEN(User!AF47)=0,"",User!AF47)</f>
         <v/>
       </c>
-      <c r="D47" s="30"/>
+      <c r="D47" s="11"/>
       <c r="E47" s="12"/>
       <c r="F47" s="12"/>
       <c r="G47" s="11"/>
@@ -4720,8 +4766,9 @@
       <c r="M47" s="12"/>
       <c r="N47" s="12"/>
       <c r="O47" s="11"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P47" s="11"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" s="12">
         <v>47</v>
       </c>
@@ -4733,7 +4780,7 @@
         <f>IF(LEN(User!AF48)=0,"",User!AF48)</f>
         <v/>
       </c>
-      <c r="D48" s="31"/>
+      <c r="D48" s="27"/>
       <c r="E48" s="12"/>
       <c r="F48" s="12"/>
       <c r="G48" s="11"/>
@@ -4748,8 +4795,9 @@
       <c r="M48" s="12"/>
       <c r="N48" s="12"/>
       <c r="O48" s="11"/>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P48" s="11"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" s="12">
         <v>48</v>
       </c>
@@ -4761,7 +4809,7 @@
         <f>IF(LEN(User!AF49)=0,"",User!AF49)</f>
         <v/>
       </c>
-      <c r="D49" s="31"/>
+      <c r="D49" s="27"/>
       <c r="E49" s="12"/>
       <c r="F49" s="12"/>
       <c r="G49" s="11"/>
@@ -4776,8 +4824,9 @@
       <c r="M49" s="12"/>
       <c r="N49" s="12"/>
       <c r="O49" s="11"/>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P49" s="11"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" s="12">
         <v>49</v>
       </c>
@@ -4789,7 +4838,7 @@
         <f>IF(LEN(User!AF50)=0,"",User!AF50)</f>
         <v/>
       </c>
-      <c r="D50" s="31"/>
+      <c r="D50" s="27"/>
       <c r="E50" s="12"/>
       <c r="F50" s="12"/>
       <c r="G50" s="11"/>
@@ -4804,8 +4853,9 @@
       <c r="M50" s="12"/>
       <c r="N50" s="12"/>
       <c r="O50" s="11"/>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="P50" s="11"/>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" s="20">
         <v>50</v>
       </c>
@@ -4817,18 +4867,19 @@
         <f>IF(LEN(User!AF51)=0,"",User!AF51)</f>
         <v/>
       </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="8"/>
-      <c r="L51" s="29"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="17"/>
+      <c r="L51" s="44"/>
       <c r="M51" s="20"/>
       <c r="N51" s="20"/>
       <c r="O51" s="21"/>
+      <c r="P51" s="21"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>

<commit_message>
NonCondition instead of NonSample
</commit_message>
<xml_diff>
--- a/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
+++ b/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/metadata_capture/excel_utils/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961FA26B-ACD6-344F-A814-E194BA40C5D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C245489-A6BF-6143-949B-688485CAE2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" activeTab="1" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -204,15 +204,6 @@
     <t>Provide one location of an empty well on any plate (e.g. RA1)</t>
   </si>
   <si>
-    <t>NonCondition at start:</t>
-  </si>
-  <si>
-    <t>NonCondition at end:</t>
-  </si>
-  <si>
-    <t>NonCondition between:</t>
-  </si>
-  <si>
     <t>For 2 column, "ChannelA_" or "ChannelB_" is added before column K (LC method file name)</t>
   </si>
   <si>
@@ -226,6 +217,15 @@
   </si>
   <si>
     <t>NonCondition Ordering: QC-&gt;Blank-&gt;Trueblank</t>
+  </si>
+  <si>
+    <t>Ending NonCondition at end:</t>
+  </si>
+  <si>
+    <t>Beginning NonCondition:</t>
+  </si>
+  <si>
+    <t>Between NonCondition:</t>
   </si>
 </sst>
 </file>
@@ -557,6 +557,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -577,12 +583,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1002,10 +1002,10 @@
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
       <c r="AO3" s="30"/>
-      <c r="AU3" s="44" t="s">
+      <c r="AU3" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="AV3" s="44"/>
+      <c r="AV3" s="46"/>
     </row>
     <row r="4" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -1045,15 +1045,15 @@
         <v>33</v>
       </c>
       <c r="AJ4" s="6"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
       <c r="AO4" s="30"/>
-      <c r="AU4" s="44"/>
-      <c r="AV4" s="44"/>
+      <c r="AU4" s="46"/>
+      <c r="AV4" s="46"/>
     </row>
     <row r="5" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
@@ -1147,15 +1147,15 @@
         <v>53</v>
       </c>
       <c r="AJ5" s="6"/>
-      <c r="AK5" s="49" t="s">
+      <c r="AK5" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="AL5" s="50"/>
+      <c r="AL5" s="52"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
       <c r="AO5" s="30"/>
-      <c r="AU5" s="44"/>
-      <c r="AV5" s="44"/>
+      <c r="AU5" s="46"/>
+      <c r="AV5" s="46"/>
     </row>
     <row r="6" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A6" s="41" t="s">
@@ -1199,8 +1199,8 @@
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
       <c r="AO6" s="30"/>
-      <c r="AU6" s="44"/>
-      <c r="AV6" s="44"/>
+      <c r="AU6" s="46"/>
+      <c r="AV6" s="46"/>
     </row>
     <row r="7" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
@@ -1239,8 +1239,8 @@
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
       <c r="AO7" s="30"/>
-      <c r="AU7" s="44"/>
-      <c r="AV7" s="44"/>
+      <c r="AU7" s="46"/>
+      <c r="AV7" s="46"/>
     </row>
     <row r="8" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
@@ -1282,15 +1282,15 @@
       <c r="AJ8" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="AK8" s="49" t="s">
+      <c r="AK8" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="AL8" s="50"/>
+      <c r="AL8" s="52"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
       <c r="AO8" s="30"/>
-      <c r="AU8" s="44"/>
-      <c r="AV8" s="44"/>
+      <c r="AU8" s="46"/>
+      <c r="AV8" s="46"/>
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D9" t="s">
@@ -1330,13 +1330,13 @@
         <v>52</v>
       </c>
       <c r="AJ9" s="6"/>
-      <c r="AK9" s="49"/>
-      <c r="AL9" s="50"/>
+      <c r="AK9" s="51"/>
+      <c r="AL9" s="52"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
       <c r="AO9" s="30"/>
-      <c r="AU9" s="44"/>
-      <c r="AV9" s="44"/>
+      <c r="AU9" s="46"/>
+      <c r="AV9" s="46"/>
     </row>
     <row r="10" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
@@ -1372,19 +1372,19 @@
       <c r="AE10" s="8"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="29"/>
-      <c r="AI10" s="45" t="s">
+      <c r="AI10" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="AJ10" s="47" t="s">
+      <c r="AJ10" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="AK10" s="49"/>
-      <c r="AL10" s="50"/>
+      <c r="AK10" s="51"/>
+      <c r="AL10" s="52"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
       <c r="AO10" s="30"/>
-      <c r="AU10" s="44"/>
-      <c r="AV10" s="44"/>
+      <c r="AU10" s="46"/>
+      <c r="AV10" s="46"/>
     </row>
     <row r="11" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D11" t="s">
@@ -1420,15 +1420,15 @@
       <c r="AE11" s="8"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="29"/>
-      <c r="AI11" s="46"/>
-      <c r="AJ11" s="48"/>
+      <c r="AI11" s="48"/>
+      <c r="AJ11" s="50"/>
       <c r="AK11" s="32"/>
       <c r="AL11" s="32"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
       <c r="AO11" s="30"/>
-      <c r="AU11" s="44"/>
-      <c r="AV11" s="44"/>
+      <c r="AU11" s="46"/>
+      <c r="AV11" s="46"/>
     </row>
     <row r="12" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
@@ -1471,8 +1471,8 @@
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
       <c r="AO12" s="30"/>
-      <c r="AU12" s="44"/>
-      <c r="AV12" s="44"/>
+      <c r="AU12" s="46"/>
+      <c r="AV12" s="46"/>
     </row>
     <row r="13" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D13" t="s">
@@ -1515,8 +1515,8 @@
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
       <c r="AO13" s="30"/>
-      <c r="AU13" s="44"/>
-      <c r="AV13" s="44"/>
+      <c r="AU13" s="46"/>
+      <c r="AV13" s="46"/>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D14" t="s">
@@ -1555,8 +1555,8 @@
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
       <c r="AO14" s="30"/>
-      <c r="AU14" s="44"/>
-      <c r="AV14" s="44"/>
+      <c r="AU14" s="46"/>
+      <c r="AV14" s="46"/>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D15" t="s">
@@ -3413,13 +3413,13 @@
         <v>9</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
@@ -3451,7 +3451,7 @@
       <c r="O2" s="11"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="34" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="R2" s="6" t="s">
         <v>43</v>
@@ -3486,7 +3486,7 @@
       <c r="O3" s="11"/>
       <c r="P3" s="11"/>
       <c r="Q3" s="38" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -3549,7 +3549,7 @@
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
       <c r="Q5" s="34" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="R5" s="6" t="s">
         <v>43</v>
@@ -3583,10 +3583,10 @@
       <c r="N6" s="12"/>
       <c r="O6" s="11"/>
       <c r="P6" s="11"/>
-      <c r="Q6" s="52" t="s">
-        <v>61</v>
-      </c>
-      <c r="R6" s="51"/>
+      <c r="Q6" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="R6" s="45"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
@@ -3712,7 +3712,7 @@
       <c r="O10" s="11"/>
       <c r="P10" s="11"/>
       <c r="Q10" s="42" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R10" s="43"/>
     </row>

</xml_diff>

<commit_message>
added 4 plates and solvent vials
</commit_message>
<xml_diff>
--- a/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
+++ b/metadata_capture/excel_utils/templates/worklist_template_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/metadata_capture/excel_utils/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C245489-A6BF-6143-949B-688485CAE2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8AD6EE-9F26-6549-8377-F67B3939FAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
+    <workbookView xWindow="14680" yWindow="700" windowWidth="14720" windowHeight="16920" activeTab="1" xr2:uid="{12DA0CF9-A1F3-4B47-B73A-18ED55D7EBC7}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="70">
   <si>
     <t>Number:</t>
   </si>
@@ -226,6 +226,27 @@
   </si>
   <si>
     <t>Between NonCondition:</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Solvent Vials</t>
+  </si>
+  <si>
+    <t>Plate 4</t>
+  </si>
+  <si>
+    <t>Injection volume:</t>
+  </si>
+  <si>
+    <t>What MS system are you using?</t>
+  </si>
+  <si>
+    <t>This determines if the run number is included at the end of each file name</t>
+  </si>
+  <si>
+    <t>System configuration:</t>
   </si>
 </sst>
 </file>
@@ -467,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
@@ -551,18 +572,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -584,6 +593,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -918,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4A45856-9C0F-D140-AD60-2AFFFFA45290}">
-  <dimension ref="A1:AV63"/>
+  <dimension ref="A1:AV76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -1002,10 +1026,10 @@
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
       <c r="AO3" s="30"/>
-      <c r="AU3" s="46" t="s">
+      <c r="AU3" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="AV3" s="46"/>
+      <c r="AV3" s="42"/>
     </row>
     <row r="4" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -1045,15 +1069,15 @@
         <v>33</v>
       </c>
       <c r="AJ4" s="6"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AK4" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="48"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
       <c r="AO4" s="30"/>
-      <c r="AU4" s="46"/>
-      <c r="AV4" s="46"/>
+      <c r="AU4" s="42"/>
+      <c r="AV4" s="42"/>
     </row>
     <row r="5" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
@@ -1147,15 +1171,15 @@
         <v>53</v>
       </c>
       <c r="AJ5" s="6"/>
-      <c r="AK5" s="51" t="s">
+      <c r="AK5" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="AL5" s="52"/>
+      <c r="AL5" s="48"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
       <c r="AO5" s="30"/>
-      <c r="AU5" s="46"/>
-      <c r="AV5" s="46"/>
+      <c r="AU5" s="42"/>
+      <c r="AV5" s="42"/>
     </row>
     <row r="6" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A6" s="41" t="s">
@@ -1199,8 +1223,8 @@
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
       <c r="AO6" s="30"/>
-      <c r="AU6" s="46"/>
-      <c r="AV6" s="46"/>
+      <c r="AU6" s="42"/>
+      <c r="AV6" s="42"/>
     </row>
     <row r="7" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
@@ -1239,8 +1263,8 @@
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
       <c r="AO7" s="30"/>
-      <c r="AU7" s="46"/>
-      <c r="AV7" s="46"/>
+      <c r="AU7" s="42"/>
+      <c r="AV7" s="42"/>
     </row>
     <row r="8" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
@@ -1282,17 +1306,20 @@
       <c r="AJ8" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="AK8" s="51" t="s">
+      <c r="AK8" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="AL8" s="52"/>
+      <c r="AL8" s="48"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
       <c r="AO8" s="30"/>
-      <c r="AU8" s="46"/>
-      <c r="AV8" s="46"/>
+      <c r="AU8" s="42"/>
+      <c r="AV8" s="42"/>
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="B9" s="31" t="s">
+        <v>64</v>
+      </c>
       <c r="D9" t="s">
         <v>16</v>
       </c>
@@ -1330,15 +1357,19 @@
         <v>52</v>
       </c>
       <c r="AJ9" s="6"/>
-      <c r="AK9" s="51"/>
-      <c r="AL9" s="52"/>
+      <c r="AK9" s="47"/>
+      <c r="AL9" s="48"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
       <c r="AO9" s="30"/>
-      <c r="AU9" s="46"/>
-      <c r="AV9" s="46"/>
+      <c r="AU9" s="42"/>
+      <c r="AV9" s="42"/>
     </row>
     <row r="10" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" s="11"/>
       <c r="D10" t="s">
         <v>17</v>
       </c>
@@ -1372,21 +1403,25 @@
       <c r="AE10" s="8"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="29"/>
-      <c r="AI10" s="47" t="s">
+      <c r="AI10" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="AJ10" s="49" t="s">
+      <c r="AJ10" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="AK10" s="51"/>
-      <c r="AL10" s="52"/>
+      <c r="AK10" s="47"/>
+      <c r="AL10" s="48"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
       <c r="AO10" s="30"/>
-      <c r="AU10" s="46"/>
-      <c r="AV10" s="46"/>
+      <c r="AU10" s="42"/>
+      <c r="AV10" s="42"/>
     </row>
     <row r="11" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" s="11"/>
       <c r="D11" t="s">
         <v>18</v>
       </c>
@@ -1420,17 +1455,21 @@
       <c r="AE11" s="8"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="29"/>
-      <c r="AI11" s="48"/>
-      <c r="AJ11" s="50"/>
+      <c r="AI11" s="44"/>
+      <c r="AJ11" s="46"/>
       <c r="AK11" s="32"/>
       <c r="AL11" s="32"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
       <c r="AO11" s="30"/>
-      <c r="AU11" s="46"/>
-      <c r="AV11" s="46"/>
+      <c r="AU11" s="42"/>
+      <c r="AV11" s="42"/>
     </row>
     <row r="12" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" s="11"/>
       <c r="D12" t="s">
         <v>19</v>
       </c>
@@ -1471,10 +1510,14 @@
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
       <c r="AO12" s="30"/>
-      <c r="AU12" s="46"/>
-      <c r="AV12" s="46"/>
+      <c r="AU12" s="42"/>
+      <c r="AV12" s="42"/>
     </row>
     <row r="13" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" s="11"/>
       <c r="D13" t="s">
         <v>20</v>
       </c>
@@ -1515,10 +1558,14 @@
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
       <c r="AO13" s="30"/>
-      <c r="AU13" s="46"/>
-      <c r="AV13" s="46"/>
+      <c r="AU13" s="42"/>
+      <c r="AV13" s="42"/>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" s="21"/>
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1555,8 +1602,8 @@
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
       <c r="AO14" s="30"/>
-      <c r="AU14" s="46"/>
-      <c r="AV14" s="46"/>
+      <c r="AU14" s="42"/>
+      <c r="AV14" s="42"/>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D15" t="s">
@@ -2109,6 +2156,9 @@
       <c r="AO26" s="30"/>
     </row>
     <row r="27" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B27" s="31" t="s">
+        <v>64</v>
+      </c>
       <c r="D27" t="s">
         <v>16</v>
       </c>
@@ -2151,6 +2201,10 @@
       <c r="AO27" s="30"/>
     </row>
     <row r="28" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" s="11"/>
       <c r="D28" t="s">
         <v>17</v>
       </c>
@@ -2193,6 +2247,10 @@
       <c r="AO28" s="30"/>
     </row>
     <row r="29" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>2</v>
+      </c>
+      <c r="B29" s="11"/>
       <c r="D29" t="s">
         <v>18</v>
       </c>
@@ -2235,6 +2293,10 @@
       <c r="AO29" s="30"/>
     </row>
     <row r="30" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>3</v>
+      </c>
+      <c r="B30" s="11"/>
       <c r="D30" t="s">
         <v>19</v>
       </c>
@@ -2277,6 +2339,10 @@
       <c r="AO30" s="30"/>
     </row>
     <row r="31" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31" s="11"/>
       <c r="D31" t="s">
         <v>20</v>
       </c>
@@ -2319,6 +2385,10 @@
       <c r="AO31" s="30"/>
     </row>
     <row r="32" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>5</v>
+      </c>
+      <c r="B32" s="21"/>
       <c r="D32" t="s">
         <v>21</v>
       </c>
@@ -2846,6 +2916,9 @@
       <c r="AG44" s="11"/>
     </row>
     <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="31" t="s">
+        <v>64</v>
+      </c>
       <c r="D45" t="s">
         <v>16</v>
       </c>
@@ -2881,6 +2954,10 @@
       <c r="AG45" s="11"/>
     </row>
     <row r="46" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" s="11"/>
       <c r="D46" t="s">
         <v>17</v>
       </c>
@@ -2916,6 +2993,10 @@
       <c r="AG46" s="11"/>
     </row>
     <row r="47" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>2</v>
+      </c>
+      <c r="B47" s="11"/>
       <c r="D47" t="s">
         <v>18</v>
       </c>
@@ -2951,6 +3032,10 @@
       <c r="AG47" s="11"/>
     </row>
     <row r="48" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="B48" s="11"/>
       <c r="D48" t="s">
         <v>19</v>
       </c>
@@ -2986,6 +3071,10 @@
       <c r="AG48" s="11"/>
     </row>
     <row r="49" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>4</v>
+      </c>
+      <c r="B49" s="11"/>
       <c r="D49" t="s">
         <v>20</v>
       </c>
@@ -3021,6 +3110,10 @@
       <c r="AG49" s="11"/>
     </row>
     <row r="50" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>5</v>
+      </c>
+      <c r="B50" s="21"/>
       <c r="D50" t="s">
         <v>21</v>
       </c>
@@ -3317,6 +3410,87 @@
       <c r="AN58" s="23"/>
     </row>
     <row r="59" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>65</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59">
+        <v>2</v>
+      </c>
+      <c r="G59">
+        <v>3</v>
+      </c>
+      <c r="H59">
+        <v>4</v>
+      </c>
+      <c r="I59">
+        <v>5</v>
+      </c>
+      <c r="J59">
+        <v>6</v>
+      </c>
+      <c r="K59">
+        <v>7</v>
+      </c>
+      <c r="L59">
+        <v>8</v>
+      </c>
+      <c r="M59">
+        <v>9</v>
+      </c>
+      <c r="N59">
+        <v>10</v>
+      </c>
+      <c r="O59">
+        <v>11</v>
+      </c>
+      <c r="P59">
+        <v>12</v>
+      </c>
+      <c r="Q59">
+        <v>13</v>
+      </c>
+      <c r="R59">
+        <v>14</v>
+      </c>
+      <c r="S59">
+        <v>15</v>
+      </c>
+      <c r="T59">
+        <v>16</v>
+      </c>
+      <c r="U59">
+        <v>17</v>
+      </c>
+      <c r="V59">
+        <v>18</v>
+      </c>
+      <c r="W59">
+        <v>19</v>
+      </c>
+      <c r="X59">
+        <v>20</v>
+      </c>
+      <c r="Y59">
+        <v>21</v>
+      </c>
+      <c r="Z59">
+        <v>22</v>
+      </c>
+      <c r="AA59">
+        <v>23</v>
+      </c>
+      <c r="AB59">
+        <v>24</v>
+      </c>
       <c r="AE59" s="10"/>
       <c r="AK59" s="23"/>
       <c r="AL59" s="24"/>
@@ -3324,16 +3498,528 @@
       <c r="AN59" s="23"/>
     </row>
     <row r="60" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A60" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" s="13"/>
+      <c r="D60" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" s="14"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
+      <c r="K60" s="15"/>
+      <c r="L60" s="15"/>
+      <c r="M60" s="15"/>
+      <c r="N60" s="15"/>
+      <c r="O60" s="15"/>
+      <c r="P60" s="15"/>
+      <c r="Q60" s="15"/>
+      <c r="R60" s="15"/>
+      <c r="S60" s="15"/>
+      <c r="T60" s="15"/>
+      <c r="U60" s="15"/>
+      <c r="V60" s="15"/>
+      <c r="W60" s="15"/>
+      <c r="X60" s="15"/>
+      <c r="Y60" s="15"/>
+      <c r="Z60" s="15"/>
+      <c r="AA60" s="15"/>
+      <c r="AB60" s="16"/>
       <c r="AE60" s="10"/>
     </row>
     <row r="61" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="D61" t="s">
+        <v>14</v>
+      </c>
+      <c r="E61" s="8"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="10"/>
+      <c r="J61" s="10"/>
+      <c r="K61" s="10"/>
+      <c r="L61" s="10"/>
+      <c r="M61" s="10"/>
+      <c r="N61" s="10"/>
+      <c r="O61" s="10"/>
+      <c r="P61" s="10"/>
+      <c r="Q61" s="10"/>
+      <c r="R61" s="10"/>
+      <c r="S61" s="10"/>
+      <c r="T61" s="10"/>
+      <c r="U61" s="10"/>
+      <c r="V61" s="10"/>
+      <c r="W61" s="10"/>
+      <c r="X61" s="10"/>
+      <c r="Y61" s="10"/>
+      <c r="Z61" s="10"/>
+      <c r="AA61" s="10"/>
+      <c r="AB61" s="9"/>
       <c r="AE61" s="10"/>
     </row>
     <row r="62" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="D62" t="s">
+        <v>15</v>
+      </c>
+      <c r="E62" s="8"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="10"/>
+      <c r="H62" s="10"/>
+      <c r="I62" s="10"/>
+      <c r="J62" s="10"/>
+      <c r="K62" s="10"/>
+      <c r="L62" s="10"/>
+      <c r="M62" s="10"/>
+      <c r="N62" s="10"/>
+      <c r="O62" s="10"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="10"/>
+      <c r="R62" s="10"/>
+      <c r="S62" s="10"/>
+      <c r="T62" s="10"/>
+      <c r="U62" s="10"/>
+      <c r="V62" s="10"/>
+      <c r="W62" s="10"/>
+      <c r="X62" s="10"/>
+      <c r="Y62" s="10"/>
+      <c r="Z62" s="10"/>
+      <c r="AA62" s="10"/>
+      <c r="AB62" s="9"/>
       <c r="AE62" s="10"/>
     </row>
     <row r="63" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="B63" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="D63" t="s">
+        <v>16</v>
+      </c>
+      <c r="E63" s="8"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+      <c r="I63" s="10"/>
+      <c r="J63" s="10"/>
+      <c r="K63" s="10"/>
+      <c r="L63" s="10"/>
+      <c r="M63" s="10"/>
+      <c r="N63" s="10"/>
+      <c r="O63" s="10"/>
+      <c r="P63" s="10"/>
+      <c r="Q63" s="10"/>
+      <c r="R63" s="10"/>
+      <c r="S63" s="10"/>
+      <c r="T63" s="10"/>
+      <c r="U63" s="10"/>
+      <c r="V63" s="10"/>
+      <c r="W63" s="10"/>
+      <c r="X63" s="10"/>
+      <c r="Y63" s="10"/>
+      <c r="Z63" s="10"/>
+      <c r="AA63" s="10"/>
+      <c r="AB63" s="9"/>
       <c r="AE63" s="10"/>
+    </row>
+    <row r="64" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>1</v>
+      </c>
+      <c r="B64" s="11"/>
+      <c r="D64" t="s">
+        <v>17</v>
+      </c>
+      <c r="E64" s="8"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+      <c r="I64" s="10"/>
+      <c r="J64" s="10"/>
+      <c r="K64" s="10"/>
+      <c r="L64" s="10"/>
+      <c r="M64" s="10"/>
+      <c r="N64" s="10"/>
+      <c r="O64" s="10"/>
+      <c r="P64" s="10"/>
+      <c r="Q64" s="10"/>
+      <c r="R64" s="10"/>
+      <c r="S64" s="10"/>
+      <c r="T64" s="10"/>
+      <c r="U64" s="10"/>
+      <c r="V64" s="10"/>
+      <c r="W64" s="10"/>
+      <c r="X64" s="10"/>
+      <c r="Y64" s="10"/>
+      <c r="Z64" s="10"/>
+      <c r="AA64" s="10"/>
+      <c r="AB64" s="9"/>
+    </row>
+    <row r="65" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>2</v>
+      </c>
+      <c r="B65" s="11"/>
+      <c r="D65" t="s">
+        <v>18</v>
+      </c>
+      <c r="E65" s="8"/>
+      <c r="F65" s="10"/>
+      <c r="G65" s="10"/>
+      <c r="H65" s="10"/>
+      <c r="I65" s="10"/>
+      <c r="J65" s="10"/>
+      <c r="K65" s="10"/>
+      <c r="L65" s="10"/>
+      <c r="M65" s="10"/>
+      <c r="N65" s="10"/>
+      <c r="O65" s="10"/>
+      <c r="P65" s="10"/>
+      <c r="Q65" s="10"/>
+      <c r="R65" s="10"/>
+      <c r="S65" s="10"/>
+      <c r="T65" s="10"/>
+      <c r="U65" s="10"/>
+      <c r="V65" s="10"/>
+      <c r="W65" s="10"/>
+      <c r="X65" s="10"/>
+      <c r="Y65" s="10"/>
+      <c r="Z65" s="10"/>
+      <c r="AA65" s="10"/>
+      <c r="AB65" s="9"/>
+    </row>
+    <row r="66" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>3</v>
+      </c>
+      <c r="B66" s="11"/>
+      <c r="D66" t="s">
+        <v>19</v>
+      </c>
+      <c r="E66" s="8"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="10"/>
+      <c r="I66" s="10"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="10"/>
+      <c r="L66" s="10"/>
+      <c r="M66" s="10"/>
+      <c r="N66" s="10"/>
+      <c r="O66" s="10"/>
+      <c r="P66" s="10"/>
+      <c r="Q66" s="10"/>
+      <c r="R66" s="10"/>
+      <c r="S66" s="10"/>
+      <c r="T66" s="10"/>
+      <c r="U66" s="10"/>
+      <c r="V66" s="10"/>
+      <c r="W66" s="10"/>
+      <c r="X66" s="10"/>
+      <c r="Y66" s="10"/>
+      <c r="Z66" s="10"/>
+      <c r="AA66" s="10"/>
+      <c r="AB66" s="9"/>
+    </row>
+    <row r="67" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>4</v>
+      </c>
+      <c r="B67" s="11"/>
+      <c r="D67" t="s">
+        <v>20</v>
+      </c>
+      <c r="E67" s="8"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="10"/>
+      <c r="I67" s="10"/>
+      <c r="J67" s="10"/>
+      <c r="K67" s="10"/>
+      <c r="L67" s="10"/>
+      <c r="M67" s="10"/>
+      <c r="N67" s="10"/>
+      <c r="O67" s="10"/>
+      <c r="P67" s="10"/>
+      <c r="Q67" s="10"/>
+      <c r="R67" s="10"/>
+      <c r="S67" s="10"/>
+      <c r="T67" s="10"/>
+      <c r="U67" s="10"/>
+      <c r="V67" s="10"/>
+      <c r="W67" s="10"/>
+      <c r="X67" s="10"/>
+      <c r="Y67" s="10"/>
+      <c r="Z67" s="10"/>
+      <c r="AA67" s="10"/>
+      <c r="AB67" s="9"/>
+    </row>
+    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>5</v>
+      </c>
+      <c r="B68" s="21"/>
+      <c r="D68" t="s">
+        <v>21</v>
+      </c>
+      <c r="E68" s="8"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+      <c r="I68" s="10"/>
+      <c r="J68" s="10"/>
+      <c r="K68" s="10"/>
+      <c r="L68" s="10"/>
+      <c r="M68" s="10"/>
+      <c r="N68" s="10"/>
+      <c r="O68" s="10"/>
+      <c r="P68" s="10"/>
+      <c r="Q68" s="10"/>
+      <c r="R68" s="10"/>
+      <c r="S68" s="10"/>
+      <c r="T68" s="10"/>
+      <c r="U68" s="10"/>
+      <c r="V68" s="10"/>
+      <c r="W68" s="10"/>
+      <c r="X68" s="10"/>
+      <c r="Y68" s="10"/>
+      <c r="Z68" s="10"/>
+      <c r="AA68" s="10"/>
+      <c r="AB68" s="9"/>
+    </row>
+    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D69" t="s">
+        <v>22</v>
+      </c>
+      <c r="E69" s="8"/>
+      <c r="F69" s="10"/>
+      <c r="G69" s="10"/>
+      <c r="H69" s="10"/>
+      <c r="I69" s="10"/>
+      <c r="J69" s="10"/>
+      <c r="K69" s="10"/>
+      <c r="L69" s="10"/>
+      <c r="M69" s="10"/>
+      <c r="N69" s="10"/>
+      <c r="O69" s="10"/>
+      <c r="P69" s="10"/>
+      <c r="Q69" s="10"/>
+      <c r="R69" s="10"/>
+      <c r="S69" s="10"/>
+      <c r="T69" s="10"/>
+      <c r="U69" s="10"/>
+      <c r="V69" s="10"/>
+      <c r="W69" s="10"/>
+      <c r="X69" s="10"/>
+      <c r="Y69" s="10"/>
+      <c r="Z69" s="10"/>
+      <c r="AA69" s="10"/>
+      <c r="AB69" s="9"/>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D70" t="s">
+        <v>23</v>
+      </c>
+      <c r="E70" s="8"/>
+      <c r="F70" s="10"/>
+      <c r="G70" s="10"/>
+      <c r="H70" s="10"/>
+      <c r="I70" s="10"/>
+      <c r="J70" s="10"/>
+      <c r="K70" s="10"/>
+      <c r="L70" s="10"/>
+      <c r="M70" s="10"/>
+      <c r="N70" s="10"/>
+      <c r="O70" s="10"/>
+      <c r="P70" s="10"/>
+      <c r="Q70" s="10"/>
+      <c r="R70" s="10"/>
+      <c r="S70" s="10"/>
+      <c r="T70" s="10"/>
+      <c r="U70" s="10"/>
+      <c r="V70" s="10"/>
+      <c r="W70" s="10"/>
+      <c r="X70" s="10"/>
+      <c r="Y70" s="10"/>
+      <c r="Z70" s="10"/>
+      <c r="AA70" s="10"/>
+      <c r="AB70" s="9"/>
+    </row>
+    <row r="71" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D71" t="s">
+        <v>24</v>
+      </c>
+      <c r="E71" s="8"/>
+      <c r="F71" s="10"/>
+      <c r="G71" s="10"/>
+      <c r="H71" s="10"/>
+      <c r="I71" s="10"/>
+      <c r="J71" s="10"/>
+      <c r="K71" s="10"/>
+      <c r="L71" s="10"/>
+      <c r="M71" s="10"/>
+      <c r="N71" s="10"/>
+      <c r="O71" s="10"/>
+      <c r="P71" s="10"/>
+      <c r="Q71" s="10"/>
+      <c r="R71" s="10"/>
+      <c r="S71" s="10"/>
+      <c r="T71" s="10"/>
+      <c r="U71" s="10"/>
+      <c r="V71" s="10"/>
+      <c r="W71" s="10"/>
+      <c r="X71" s="10"/>
+      <c r="Y71" s="10"/>
+      <c r="Z71" s="10"/>
+      <c r="AA71" s="10"/>
+      <c r="AB71" s="9"/>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D72" t="s">
+        <v>25</v>
+      </c>
+      <c r="E72" s="8"/>
+      <c r="F72" s="10"/>
+      <c r="G72" s="10"/>
+      <c r="H72" s="10"/>
+      <c r="I72" s="10"/>
+      <c r="J72" s="10"/>
+      <c r="K72" s="10"/>
+      <c r="L72" s="10"/>
+      <c r="M72" s="10"/>
+      <c r="N72" s="10"/>
+      <c r="O72" s="10"/>
+      <c r="P72" s="10"/>
+      <c r="Q72" s="10"/>
+      <c r="R72" s="10"/>
+      <c r="S72" s="10"/>
+      <c r="T72" s="10"/>
+      <c r="U72" s="10"/>
+      <c r="V72" s="10"/>
+      <c r="W72" s="10"/>
+      <c r="X72" s="10"/>
+      <c r="Y72" s="10"/>
+      <c r="Z72" s="10"/>
+      <c r="AA72" s="10"/>
+      <c r="AB72" s="9"/>
+    </row>
+    <row r="73" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D73" t="s">
+        <v>26</v>
+      </c>
+      <c r="E73" s="8"/>
+      <c r="F73" s="10"/>
+      <c r="G73" s="10"/>
+      <c r="H73" s="10"/>
+      <c r="I73" s="10"/>
+      <c r="J73" s="10"/>
+      <c r="K73" s="10"/>
+      <c r="L73" s="10"/>
+      <c r="M73" s="10"/>
+      <c r="N73" s="10"/>
+      <c r="O73" s="10"/>
+      <c r="P73" s="10"/>
+      <c r="Q73" s="10"/>
+      <c r="R73" s="10"/>
+      <c r="S73" s="10"/>
+      <c r="T73" s="10"/>
+      <c r="U73" s="10"/>
+      <c r="V73" s="10"/>
+      <c r="W73" s="10"/>
+      <c r="X73" s="10"/>
+      <c r="Y73" s="10"/>
+      <c r="Z73" s="10"/>
+      <c r="AA73" s="10"/>
+      <c r="AB73" s="9"/>
+    </row>
+    <row r="74" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D74" t="s">
+        <v>27</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="F74" s="10"/>
+      <c r="G74" s="10"/>
+      <c r="H74" s="10"/>
+      <c r="I74" s="10"/>
+      <c r="J74" s="10"/>
+      <c r="K74" s="10"/>
+      <c r="L74" s="10"/>
+      <c r="M74" s="10"/>
+      <c r="N74" s="10"/>
+      <c r="O74" s="10"/>
+      <c r="P74" s="10"/>
+      <c r="Q74" s="10"/>
+      <c r="R74" s="10"/>
+      <c r="S74" s="10"/>
+      <c r="T74" s="10"/>
+      <c r="U74" s="10"/>
+      <c r="V74" s="10"/>
+      <c r="W74" s="10"/>
+      <c r="X74" s="10"/>
+      <c r="Y74" s="10"/>
+      <c r="Z74" s="10"/>
+      <c r="AA74" s="10"/>
+      <c r="AB74" s="9"/>
+    </row>
+    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="D75" t="s">
+        <v>28</v>
+      </c>
+      <c r="E75" s="17"/>
+      <c r="F75" s="18"/>
+      <c r="G75" s="18"/>
+      <c r="H75" s="18"/>
+      <c r="I75" s="18"/>
+      <c r="J75" s="18"/>
+      <c r="K75" s="18"/>
+      <c r="L75" s="18"/>
+      <c r="M75" s="18"/>
+      <c r="N75" s="18"/>
+      <c r="O75" s="18"/>
+      <c r="P75" s="18"/>
+      <c r="Q75" s="18"/>
+      <c r="R75" s="18"/>
+      <c r="S75" s="18"/>
+      <c r="T75" s="18"/>
+      <c r="U75" s="18"/>
+      <c r="V75" s="18"/>
+      <c r="W75" s="18"/>
+      <c r="X75" s="18"/>
+      <c r="Y75" s="18"/>
+      <c r="Z75" s="18"/>
+      <c r="AA75" s="18"/>
+      <c r="AB75" s="19"/>
+    </row>
+    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="3"/>
+      <c r="P76" s="3"/>
+      <c r="Q76" s="3"/>
+      <c r="R76" s="3"/>
+      <c r="S76" s="3"/>
+      <c r="T76" s="3"/>
+      <c r="U76" s="3"/>
+      <c r="V76" s="3"/>
+      <c r="W76" s="3"/>
+      <c r="X76" s="3"/>
+      <c r="Y76" s="3"/>
+      <c r="Z76" s="3"/>
+      <c r="AA76" s="3"/>
+      <c r="AB76" s="3"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
@@ -3346,15 +4032,18 @@
     <mergeCell ref="AK5:AL5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2:AE51" xr:uid="{F021A723-187F-DD4D-8685-6A2D324FBA89}">
       <formula1>"Condition,QC,Blank,TrueBlank,Library,SystemValidation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A24 A42 A6" xr:uid="{77917AAB-E5BC-9D49-9737-341DECD5F2E8}">
-      <formula1>"R,G,B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A42 A60" xr:uid="{77917AAB-E5BC-9D49-9737-341DECD5F2E8}">
+      <formula1>"R,G,B,Y"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ4 AJ10:AJ11" xr:uid="{FA86A04D-C042-8741-AB64-AFB417F744D7}">
       <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A6 A24" xr:uid="{F1542549-AB47-124C-86A7-24ACAE350AF3}">
+      <formula1>"R,G,B,Y"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3364,15 +4053,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA40715-6F6B-5649-8058-60881427272C}">
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="17" max="17" width="30.83203125" customWidth="1"/>
-    <col min="18" max="18" width="19.6640625" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="30.83203125" customWidth="1"/>
+    <col min="19" max="19" width="19.6640625" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3413,16 +4102,22 @@
         <v>9</v>
       </c>
       <c r="N1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R1" s="55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -3448,16 +4143,17 @@
       </c>
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
-      <c r="O2" s="11"/>
+      <c r="O2" s="12"/>
       <c r="P2" s="11"/>
-      <c r="Q2" s="34" t="s">
+      <c r="Q2" s="11"/>
+      <c r="R2" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -3483,13 +4179,14 @@
       </c>
       <c r="M3" s="12"/>
       <c r="N3" s="12"/>
-      <c r="O3" s="11"/>
+      <c r="O3" s="12"/>
       <c r="P3" s="11"/>
-      <c r="Q3" s="38" t="s">
+      <c r="Q3" s="11"/>
+      <c r="R3" s="38" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -3515,12 +4212,13 @@
       </c>
       <c r="M4" s="12"/>
       <c r="N4" s="12"/>
-      <c r="O4" s="11"/>
+      <c r="O4" s="12"/>
       <c r="P4" s="11"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="24"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q4" s="11"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="24"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -3546,16 +4244,17 @@
       </c>
       <c r="M5" s="12"/>
       <c r="N5" s="12"/>
-      <c r="O5" s="11"/>
+      <c r="O5" s="12"/>
       <c r="P5" s="11"/>
-      <c r="Q5" s="34" t="s">
+      <c r="Q5" s="11"/>
+      <c r="R5" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="S5" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -3581,14 +4280,15 @@
       </c>
       <c r="M6" s="12"/>
       <c r="N6" s="12"/>
-      <c r="O6" s="11"/>
+      <c r="O6" s="12"/>
       <c r="P6" s="11"/>
-      <c r="Q6" s="44" t="s">
+      <c r="Q6" s="11"/>
+      <c r="R6" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="R6" s="45"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S6" s="52"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -3614,10 +4314,11 @@
       </c>
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
-      <c r="O7" s="11"/>
+      <c r="O7" s="12"/>
       <c r="P7" s="11"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q7" s="11"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -3643,14 +4344,15 @@
       </c>
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
-      <c r="O8" s="11"/>
+      <c r="O8" s="12"/>
       <c r="P8" s="11"/>
-      <c r="Q8" s="35" t="s">
+      <c r="Q8" s="11"/>
+      <c r="R8" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="R8" s="6"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S8" s="6"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -3676,14 +4378,15 @@
       </c>
       <c r="M9" s="12"/>
       <c r="N9" s="12"/>
-      <c r="O9" s="11"/>
+      <c r="O9" s="12"/>
       <c r="P9" s="11"/>
-      <c r="Q9" s="1" t="s">
+      <c r="Q9" s="11"/>
+      <c r="R9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="R9" s="6"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S9" s="6"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -3709,14 +4412,15 @@
       </c>
       <c r="M10" s="12"/>
       <c r="N10" s="12"/>
-      <c r="O10" s="11"/>
+      <c r="O10" s="12"/>
       <c r="P10" s="11"/>
-      <c r="Q10" s="42" t="s">
+      <c r="Q10" s="11"/>
+      <c r="R10" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="R10" s="43"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S10" s="50"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="12">
         <v>10</v>
       </c>
@@ -3742,10 +4446,11 @@
       </c>
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
-      <c r="O11" s="11"/>
+      <c r="O11" s="12"/>
       <c r="P11" s="11"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q11" s="11"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -3771,16 +4476,17 @@
       </c>
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
-      <c r="O12" s="11"/>
+      <c r="O12" s="12"/>
       <c r="P12" s="11"/>
-      <c r="Q12" s="1" t="s">
+      <c r="Q12" s="11"/>
+      <c r="R12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R12" s="6" t="s">
+      <c r="S12" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -3806,14 +4512,15 @@
       </c>
       <c r="M13" s="12"/>
       <c r="N13" s="12"/>
-      <c r="O13" s="11"/>
+      <c r="O13" s="12"/>
       <c r="P13" s="11"/>
-      <c r="Q13" s="42" t="s">
+      <c r="Q13" s="11"/>
+      <c r="R13" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="R13" s="43"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S13" s="50"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -3839,10 +4546,17 @@
       </c>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="11"/>
+      <c r="O14" s="12"/>
       <c r="P14" s="11"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="Q14" s="11"/>
+      <c r="R14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -3868,10 +4582,15 @@
       </c>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
-      <c r="O15" s="11"/>
+      <c r="O15" s="12"/>
       <c r="P15" s="11"/>
-    </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q15" s="11"/>
+      <c r="R15" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="S15" s="54"/>
+    </row>
+    <row r="16" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -3897,10 +4616,11 @@
       </c>
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
-      <c r="O16" s="11"/>
+      <c r="O16" s="12"/>
       <c r="P16" s="11"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q16" s="11"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -3926,10 +4646,11 @@
       </c>
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
-      <c r="O17" s="11"/>
+      <c r="O17" s="12"/>
       <c r="P17" s="11"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q17" s="11"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="12">
         <v>17</v>
       </c>
@@ -3955,10 +4676,11 @@
       </c>
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
-      <c r="O18" s="11"/>
+      <c r="O18" s="12"/>
       <c r="P18" s="11"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q18" s="11"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" s="12">
         <v>18</v>
       </c>
@@ -3984,10 +4706,11 @@
       </c>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
-      <c r="O19" s="11"/>
+      <c r="O19" s="12"/>
       <c r="P19" s="11"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q19" s="11"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" s="12">
         <v>19</v>
       </c>
@@ -4013,10 +4736,11 @@
       </c>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
-      <c r="O20" s="11"/>
+      <c r="O20" s="12"/>
       <c r="P20" s="11"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q20" s="11"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" s="12">
         <v>20</v>
       </c>
@@ -4042,10 +4766,11 @@
       </c>
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
-      <c r="O21" s="11"/>
+      <c r="O21" s="12"/>
       <c r="P21" s="11"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q21" s="11"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="12">
         <v>21</v>
       </c>
@@ -4071,10 +4796,11 @@
       </c>
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
-      <c r="O22" s="11"/>
+      <c r="O22" s="12"/>
       <c r="P22" s="11"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q22" s="11"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" s="12">
         <v>22</v>
       </c>
@@ -4100,10 +4826,11 @@
       </c>
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
-      <c r="O23" s="11"/>
+      <c r="O23" s="12"/>
       <c r="P23" s="11"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q23" s="11"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -4129,10 +4856,11 @@
       </c>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
-      <c r="O24" s="11"/>
+      <c r="O24" s="12"/>
       <c r="P24" s="11"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q24" s="11"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -4158,10 +4886,11 @@
       </c>
       <c r="M25" s="12"/>
       <c r="N25" s="12"/>
-      <c r="O25" s="11"/>
+      <c r="O25" s="12"/>
       <c r="P25" s="11"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q25" s="11"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" s="12">
         <v>25</v>
       </c>
@@ -4187,10 +4916,11 @@
       </c>
       <c r="M26" s="12"/>
       <c r="N26" s="12"/>
-      <c r="O26" s="11"/>
+      <c r="O26" s="12"/>
       <c r="P26" s="11"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q26" s="11"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" s="12">
         <v>26</v>
       </c>
@@ -4216,10 +4946,11 @@
       </c>
       <c r="M27" s="12"/>
       <c r="N27" s="12"/>
-      <c r="O27" s="11"/>
+      <c r="O27" s="12"/>
       <c r="P27" s="11"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q27" s="11"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" s="12">
         <v>27</v>
       </c>
@@ -4245,10 +4976,11 @@
       </c>
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
-      <c r="O28" s="11"/>
+      <c r="O28" s="12"/>
       <c r="P28" s="11"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q28" s="11"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -4274,10 +5006,11 @@
       </c>
       <c r="M29" s="12"/>
       <c r="N29" s="12"/>
-      <c r="O29" s="11"/>
+      <c r="O29" s="12"/>
       <c r="P29" s="11"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q29" s="11"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" s="12">
         <v>29</v>
       </c>
@@ -4303,10 +5036,11 @@
       </c>
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
-      <c r="O30" s="11"/>
+      <c r="O30" s="12"/>
       <c r="P30" s="11"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q30" s="11"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" s="12">
         <v>30</v>
       </c>
@@ -4332,10 +5066,11 @@
       </c>
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
-      <c r="O31" s="11"/>
+      <c r="O31" s="12"/>
       <c r="P31" s="11"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q31" s="11"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" s="12">
         <v>31</v>
       </c>
@@ -4361,10 +5096,11 @@
       </c>
       <c r="M32" s="12"/>
       <c r="N32" s="12"/>
-      <c r="O32" s="11"/>
+      <c r="O32" s="12"/>
       <c r="P32" s="11"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q32" s="11"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="12">
         <v>32</v>
       </c>
@@ -4390,10 +5126,11 @@
       </c>
       <c r="M33" s="12"/>
       <c r="N33" s="12"/>
-      <c r="O33" s="11"/>
+      <c r="O33" s="12"/>
       <c r="P33" s="11"/>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q33" s="11"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" s="12">
         <v>33</v>
       </c>
@@ -4419,10 +5156,11 @@
       </c>
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
-      <c r="O34" s="11"/>
+      <c r="O34" s="12"/>
       <c r="P34" s="11"/>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q34" s="11"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" s="12">
         <v>34</v>
       </c>
@@ -4448,10 +5186,11 @@
       </c>
       <c r="M35" s="12"/>
       <c r="N35" s="12"/>
-      <c r="O35" s="11"/>
+      <c r="O35" s="12"/>
       <c r="P35" s="11"/>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q35" s="11"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="12">
         <v>35</v>
       </c>
@@ -4475,11 +5214,12 @@
         <f>IF(LEN(User!AG36)=0,"",User!AG36)</f>
         <v/>
       </c>
-      <c r="N36" s="12"/>
-      <c r="O36" s="11"/>
+      <c r="M36" s="11"/>
+      <c r="O36" s="12"/>
       <c r="P36" s="11"/>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q36" s="11"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" s="12">
         <v>36</v>
       </c>
@@ -4505,10 +5245,11 @@
       </c>
       <c r="M37" s="12"/>
       <c r="N37" s="12"/>
-      <c r="O37" s="11"/>
+      <c r="O37" s="12"/>
       <c r="P37" s="11"/>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q37" s="11"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" s="12">
         <v>37</v>
       </c>
@@ -4534,10 +5275,11 @@
       </c>
       <c r="M38" s="12"/>
       <c r="N38" s="12"/>
-      <c r="O38" s="11"/>
+      <c r="O38" s="12"/>
       <c r="P38" s="11"/>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q38" s="11"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" s="12">
         <v>38</v>
       </c>
@@ -4563,10 +5305,11 @@
       </c>
       <c r="M39" s="12"/>
       <c r="N39" s="12"/>
-      <c r="O39" s="11"/>
+      <c r="O39" s="12"/>
       <c r="P39" s="11"/>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q39" s="11"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="12">
         <v>39</v>
       </c>
@@ -4592,10 +5335,11 @@
       </c>
       <c r="M40" s="12"/>
       <c r="N40" s="12"/>
-      <c r="O40" s="11"/>
+      <c r="O40" s="12"/>
       <c r="P40" s="11"/>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q40" s="11"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="12">
         <v>40</v>
       </c>
@@ -4621,10 +5365,11 @@
       </c>
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
-      <c r="O41" s="11"/>
+      <c r="O41" s="12"/>
       <c r="P41" s="11"/>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q41" s="11"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="12">
         <v>41</v>
       </c>
@@ -4650,10 +5395,11 @@
       </c>
       <c r="M42" s="12"/>
       <c r="N42" s="12"/>
-      <c r="O42" s="11"/>
+      <c r="O42" s="12"/>
       <c r="P42" s="11"/>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q42" s="11"/>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="12">
         <v>42</v>
       </c>
@@ -4679,10 +5425,11 @@
       </c>
       <c r="M43" s="12"/>
       <c r="N43" s="12"/>
-      <c r="O43" s="11"/>
+      <c r="O43" s="12"/>
       <c r="P43" s="11"/>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q43" s="11"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" s="12">
         <v>43</v>
       </c>
@@ -4708,10 +5455,11 @@
       </c>
       <c r="M44" s="12"/>
       <c r="N44" s="12"/>
-      <c r="O44" s="11"/>
+      <c r="O44" s="12"/>
       <c r="P44" s="11"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q44" s="11"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" s="12">
         <v>44</v>
       </c>
@@ -4737,10 +5485,11 @@
       </c>
       <c r="M45" s="12"/>
       <c r="N45" s="12"/>
-      <c r="O45" s="11"/>
+      <c r="O45" s="12"/>
       <c r="P45" s="11"/>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q45" s="11"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" s="12">
         <v>45</v>
       </c>
@@ -4766,10 +5515,11 @@
       </c>
       <c r="M46" s="12"/>
       <c r="N46" s="12"/>
-      <c r="O46" s="11"/>
+      <c r="O46" s="12"/>
       <c r="P46" s="11"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q46" s="11"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" s="12">
         <v>46</v>
       </c>
@@ -4795,10 +5545,11 @@
       </c>
       <c r="M47" s="12"/>
       <c r="N47" s="12"/>
-      <c r="O47" s="11"/>
+      <c r="O47" s="12"/>
       <c r="P47" s="11"/>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q47" s="11"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" s="12">
         <v>47</v>
       </c>
@@ -4824,10 +5575,11 @@
       </c>
       <c r="M48" s="12"/>
       <c r="N48" s="12"/>
-      <c r="O48" s="11"/>
+      <c r="O48" s="12"/>
       <c r="P48" s="11"/>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q48" s="11"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" s="12">
         <v>48</v>
       </c>
@@ -4853,10 +5605,11 @@
       </c>
       <c r="M49" s="12"/>
       <c r="N49" s="12"/>
-      <c r="O49" s="11"/>
+      <c r="O49" s="12"/>
       <c r="P49" s="11"/>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q49" s="11"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" s="12">
         <v>49</v>
       </c>
@@ -4882,10 +5635,11 @@
       </c>
       <c r="M50" s="12"/>
       <c r="N50" s="12"/>
-      <c r="O50" s="11"/>
+      <c r="O50" s="12"/>
       <c r="P50" s="11"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q50" s="11"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" s="20">
         <v>50</v>
       </c>
@@ -4908,27 +5662,31 @@
       <c r="L51" s="36"/>
       <c r="M51" s="20"/>
       <c r="N51" s="20"/>
-      <c r="O51" s="21"/>
+      <c r="O51" s="20"/>
       <c r="P51" s="21"/>
+      <c r="Q51" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="R10:S10"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:C51" xr:uid="{187E9458-F80F-4040-ADAB-CFE8AE95B8DD}">
       <formula1>"Condition,QC,Blank,TrueBlank,Lib,SystemValidation,WetQC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R5" xr:uid="{FEBF46E2-B8D0-DB4A-AFDC-F2F0CF8E04A9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S5" xr:uid="{FEBF46E2-B8D0-DB4A-AFDC-F2F0CF8E04A9}">
       <formula1>"(choose),Before,After"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2" xr:uid="{38B3635F-E371-C941-A218-633361397008}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2" xr:uid="{38B3635F-E371-C941-A218-633361397008}">
       <formula1>"(choose),1 column,2 column"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R12" xr:uid="{2E5E2557-CE3C-B44D-8B8A-511580237051}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S12" xr:uid="{2E5E2557-CE3C-B44D-8B8A-511580237051}">
       <formula1>"(choose),UltiMate3000,Vanquish Neo"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S14" xr:uid="{3AF9F873-22F8-2342-ABC0-73220D8F4575}">
+      <formula1>"(choose),Thermo,Bruker"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>